<commit_message>
updating instructions and text
</commit_message>
<xml_diff>
--- a/data/ALAI UP Client-level Reporting Tool_short_template_2.26.26.xlsx
+++ b/data/ALAI UP Client-level Reporting Tool_short_template_2.26.26.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kmlab\Desktop\Dashboard\alai_up_local_dashboard\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9C2E775-8397-434C-BD42-8BAEF941B4A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B43DA1EA-AE37-4646-AE84-1C0CCA526BFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{500E2EE0-B1C5-4ACF-BC67-EDC8BDABD2D7}"/>
+    <workbookView xWindow="-28920" yWindow="-9840" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{500E2EE0-B1C5-4ACF-BC67-EDC8BDABD2D7}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="3" r:id="rId1"/>
@@ -963,9 +963,6 @@
   </si>
   <si>
     <t>Injection 1 dose</t>
-  </si>
-  <si>
-    <t>Dose of client's first iCAB/RPV injection.</t>
   </si>
   <si>
     <t>1 = 400mg/2mL cabotegravir &amp; 600mg/2mL rilpivirine (monthly); 2 = 600mg/3mL cabotegravir &amp; 900mg/3mL rilpivirine (bimonthly); 3 = late for shot requiring reload. This is a loading dose (600mg/3mL cabotegravir &amp; 900mg/3mL rilpivirine); 4 = discontinued, restarting requiring reload. This is a loading dose (600mg/3mL CAB &amp; 900mg/3mL RPV); 5 = came or returned to clinic on CAB. Monthly maintenance dose of 400mg/2mL cabotegravir &amp; 600mg/2mL rilpivirine; 6 = came or returned to clinic on CAB. Bimonthly maintenance dose of 600mg/3mL cabotegravir &amp; 900mg/3mL rilpivirine; UNK = Unknown</t>
@@ -1967,6 +1964,10 @@
       <t xml:space="preserve">
 Please record any additional information about discontinuation and/or restarts in icab_rpv_discontinued_reason_other (e.g., client discontinued on MM/DD/YYYY due to loss of insurance but restarted at site on MM/DD/YYYY).</t>
     </r>
+  </si>
+  <si>
+    <t>Dose of client's first iCAB/RPV injection.
+Note: for icab_rpv_shot1_dose, use code 2 for a typical loading dose. The dashboard code assumes that the next dose has an injection interval of 1 month (since it is a loading dose). If the expected interval is not 1 month (e.g. if a patient came from another clinic already on monthly iCAB/RPV, use code 6.</t>
   </si>
 </sst>
 </file>
@@ -2374,7 +2375,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="132">
+  <cellXfs count="131">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -2666,7 +2667,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -3112,7 +3112,7 @@
     </row>
     <row r="7" spans="2:2" ht="27.6" x14ac:dyDescent="0.25">
       <c r="B7" s="89" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="8" spans="2:2" x14ac:dyDescent="0.25">
@@ -3122,7 +3122,7 @@
     </row>
     <row r="9" spans="2:2" ht="41.4" x14ac:dyDescent="0.25">
       <c r="B9" s="89" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
     </row>
     <row r="10" spans="2:2" x14ac:dyDescent="0.25">
@@ -3260,7 +3260,7 @@
         <v>26</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="H1" s="3"/>
       <c r="I1" s="4"/>
@@ -3268,24 +3268,24 @@
       <c r="K1" s="4"/>
     </row>
     <row r="2" spans="1:11" s="9" customFormat="1" ht="68.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="109"/>
-      <c r="B2" s="110" t="s">
+      <c r="A2"/>
+      <c r="B2" s="109" t="s">
         <v>27</v>
       </c>
-      <c r="C2" s="110" t="s">
+      <c r="C2" s="109" t="s">
         <v>28</v>
       </c>
-      <c r="D2" s="111" t="s">
+      <c r="D2" s="110" t="s">
         <v>29</v>
       </c>
-      <c r="E2" s="111" t="s">
-        <v>472</v>
-      </c>
-      <c r="F2" s="111" t="s">
+      <c r="E2" s="110" t="s">
+        <v>471</v>
+      </c>
+      <c r="F2" s="110" t="s">
         <v>30</v>
       </c>
-      <c r="G2" s="111" t="s">
-        <v>525</v>
+      <c r="G2" s="110" t="s">
+        <v>524</v>
       </c>
       <c r="H2" s="7"/>
       <c r="I2" s="8"/>
@@ -3293,24 +3293,23 @@
       <c r="K2" s="4"/>
     </row>
     <row r="3" spans="1:11" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="109"/>
       <c r="B3" s="15" t="s">
         <v>31</v>
       </c>
-      <c r="C3" s="112" t="s">
+      <c r="C3" s="111" t="s">
         <v>32</v>
       </c>
-      <c r="D3" s="113" t="s">
+      <c r="D3" s="112" t="s">
         <v>33</v>
       </c>
-      <c r="E3" s="113" t="s">
+      <c r="E3" s="112" t="s">
         <v>34</v>
       </c>
-      <c r="F3" s="113" t="s">
+      <c r="F3" s="112" t="s">
         <v>30</v>
       </c>
-      <c r="G3" s="113" t="s">
-        <v>526</v>
+      <c r="G3" s="112" t="s">
+        <v>525</v>
       </c>
       <c r="H3" s="12"/>
       <c r="I3" s="8"/>
@@ -3332,7 +3331,7 @@
         <v>38</v>
       </c>
       <c r="G4" s="16" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H4" s="12"/>
       <c r="I4" s="8"/>
@@ -3354,13 +3353,12 @@
         <v>42</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H5" s="10"/>
       <c r="I5" s="17"/>
     </row>
     <row r="6" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A6" s="109"/>
       <c r="B6" s="15" t="s">
         <v>31</v>
       </c>
@@ -3377,7 +3375,7 @@
         <v>46</v>
       </c>
       <c r="G6" s="16" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H6" s="12"/>
     </row>
@@ -3398,7 +3396,7 @@
         <v>50</v>
       </c>
       <c r="G7" s="16" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H7" s="12"/>
     </row>
@@ -3420,7 +3418,7 @@
         <v>54</v>
       </c>
       <c r="G8" s="16" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H8" s="10"/>
       <c r="I8" s="18"/>
@@ -3444,7 +3442,7 @@
         <v>58</v>
       </c>
       <c r="G9" s="16" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H9" s="12"/>
     </row>
@@ -3465,7 +3463,7 @@
         <v>62</v>
       </c>
       <c r="G10" s="16" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H10" s="12"/>
     </row>
@@ -3486,11 +3484,11 @@
         <v>66</v>
       </c>
       <c r="G11" s="16" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H11" s="12"/>
     </row>
-    <row r="12" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" ht="39.6" x14ac:dyDescent="0.3">
       <c r="B12" s="15" t="s">
         <v>31</v>
       </c>
@@ -3507,7 +3505,7 @@
         <v>70</v>
       </c>
       <c r="G12" s="16" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H12" s="12"/>
     </row>
@@ -3528,7 +3526,7 @@
         <v>74</v>
       </c>
       <c r="G13" s="16" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H13" s="12"/>
     </row>
@@ -3549,7 +3547,7 @@
         <v>78</v>
       </c>
       <c r="G14" s="16" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H14" s="12"/>
     </row>
@@ -3570,7 +3568,7 @@
         <v>30</v>
       </c>
       <c r="G15" s="16" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H15" s="12"/>
     </row>
@@ -3591,11 +3589,11 @@
         <v>85</v>
       </c>
       <c r="G16" s="16" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H16" s="20"/>
     </row>
-    <row r="17" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:8" ht="26.4" x14ac:dyDescent="0.3">
       <c r="B17" s="15" t="s">
         <v>31</v>
       </c>
@@ -3612,236 +3610,225 @@
         <v>89</v>
       </c>
       <c r="G17" s="16" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H17" s="12"/>
     </row>
-    <row r="18" spans="1:8" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A18" s="109"/>
-      <c r="B18" s="114" t="s">
+    <row r="18" spans="2:8" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="B18" s="113" t="s">
         <v>90</v>
       </c>
-      <c r="C18" s="114" t="s">
+      <c r="C18" s="113" t="s">
         <v>91</v>
       </c>
-      <c r="D18" s="115" t="s">
+      <c r="D18" s="114" t="s">
         <v>92</v>
       </c>
-      <c r="E18" s="115" t="s">
+      <c r="E18" s="114" t="s">
         <v>93</v>
       </c>
-      <c r="F18" s="115" t="s">
+      <c r="F18" s="114" t="s">
         <v>94</v>
       </c>
-      <c r="G18" s="115" t="s">
-        <v>528</v>
+      <c r="G18" s="114" t="s">
+        <v>527</v>
       </c>
       <c r="H18" s="12"/>
     </row>
-    <row r="19" spans="1:8" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A19" s="109"/>
-      <c r="B19" s="114" t="s">
+    <row r="19" spans="2:8" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="B19" s="113" t="s">
         <v>90</v>
       </c>
-      <c r="C19" s="114" t="s">
+      <c r="C19" s="113" t="s">
         <v>95</v>
       </c>
-      <c r="D19" s="115" t="s">
+      <c r="D19" s="114" t="s">
         <v>96</v>
       </c>
-      <c r="E19" s="115" t="s">
+      <c r="E19" s="114" t="s">
         <v>97</v>
       </c>
-      <c r="F19" s="115" t="s">
+      <c r="F19" s="114" t="s">
         <v>94</v>
       </c>
-      <c r="G19" s="115" t="s">
-        <v>528</v>
+      <c r="G19" s="114" t="s">
+        <v>527</v>
       </c>
       <c r="H19" s="12"/>
     </row>
-    <row r="20" spans="1:8" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A20" s="109"/>
-      <c r="B20" s="114" t="s">
+    <row r="20" spans="2:8" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="B20" s="113" t="s">
         <v>90</v>
       </c>
-      <c r="C20" s="114" t="s">
+      <c r="C20" s="113" t="s">
         <v>98</v>
       </c>
-      <c r="D20" s="115" t="s">
+      <c r="D20" s="114" t="s">
         <v>99</v>
       </c>
-      <c r="E20" s="115" t="s">
+      <c r="E20" s="114" t="s">
         <v>100</v>
       </c>
-      <c r="F20" s="115" t="s">
+      <c r="F20" s="114" t="s">
         <v>94</v>
       </c>
-      <c r="G20" s="115" t="s">
-        <v>528</v>
+      <c r="G20" s="114" t="s">
+        <v>527</v>
       </c>
       <c r="H20" s="12"/>
     </row>
-    <row r="21" spans="1:8" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A21" s="109"/>
-      <c r="B21" s="114" t="s">
+    <row r="21" spans="2:8" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="B21" s="113" t="s">
         <v>90</v>
       </c>
-      <c r="C21" s="114" t="s">
+      <c r="C21" s="113" t="s">
         <v>101</v>
       </c>
-      <c r="D21" s="115" t="s">
+      <c r="D21" s="114" t="s">
         <v>102</v>
       </c>
-      <c r="E21" s="115" t="s">
+      <c r="E21" s="114" t="s">
         <v>103</v>
       </c>
-      <c r="F21" s="115" t="s">
+      <c r="F21" s="114" t="s">
         <v>94</v>
       </c>
-      <c r="G21" s="115" t="s">
-        <v>528</v>
+      <c r="G21" s="114" t="s">
+        <v>527</v>
       </c>
       <c r="H21" s="12"/>
     </row>
-    <row r="22" spans="1:8" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A22" s="109"/>
-      <c r="B22" s="114" t="s">
+    <row r="22" spans="2:8" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="B22" s="113" t="s">
         <v>90</v>
       </c>
-      <c r="C22" s="114" t="s">
+      <c r="C22" s="113" t="s">
         <v>104</v>
       </c>
-      <c r="D22" s="115" t="s">
+      <c r="D22" s="114" t="s">
         <v>105</v>
       </c>
-      <c r="E22" s="115" t="s">
+      <c r="E22" s="114" t="s">
         <v>106</v>
       </c>
-      <c r="F22" s="115" t="s">
+      <c r="F22" s="114" t="s">
         <v>94</v>
       </c>
-      <c r="G22" s="115" t="s">
-        <v>528</v>
+      <c r="G22" s="114" t="s">
+        <v>527</v>
       </c>
       <c r="H22" s="12"/>
     </row>
-    <row r="23" spans="1:8" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A23" s="109"/>
-      <c r="B23" s="114" t="s">
+    <row r="23" spans="2:8" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="B23" s="113" t="s">
         <v>90</v>
       </c>
-      <c r="C23" s="114" t="s">
+      <c r="C23" s="113" t="s">
+        <v>503</v>
+      </c>
+      <c r="D23" s="114" t="s">
+        <v>508</v>
+      </c>
+      <c r="E23" s="114" t="s">
+        <v>513</v>
+      </c>
+      <c r="F23" s="114" t="s">
+        <v>94</v>
+      </c>
+      <c r="G23" s="114" t="s">
+        <v>527</v>
+      </c>
+      <c r="H23" s="12"/>
+    </row>
+    <row r="24" spans="2:8" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="B24" s="113" t="s">
+        <v>90</v>
+      </c>
+      <c r="C24" s="113" t="s">
         <v>504</v>
       </c>
-      <c r="D23" s="115" t="s">
+      <c r="D24" s="114" t="s">
         <v>509</v>
       </c>
-      <c r="E23" s="115" t="s">
+      <c r="E24" s="114" t="s">
         <v>514</v>
       </c>
-      <c r="F23" s="115" t="s">
+      <c r="F24" s="114" t="s">
         <v>94</v>
       </c>
-      <c r="G23" s="115" t="s">
-        <v>528</v>
-      </c>
-      <c r="H23" s="12"/>
-    </row>
-    <row r="24" spans="1:8" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A24" s="109"/>
-      <c r="B24" s="114" t="s">
+      <c r="G24" s="114" t="s">
+        <v>527</v>
+      </c>
+      <c r="H24" s="12"/>
+    </row>
+    <row r="25" spans="2:8" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="B25" s="113" t="s">
         <v>90</v>
       </c>
-      <c r="C24" s="114" t="s">
+      <c r="C25" s="113" t="s">
         <v>505</v>
       </c>
-      <c r="D24" s="115" t="s">
+      <c r="D25" s="114" t="s">
         <v>510</v>
       </c>
-      <c r="E24" s="115" t="s">
+      <c r="E25" s="114" t="s">
         <v>515</v>
       </c>
-      <c r="F24" s="115" t="s">
+      <c r="F25" s="114" t="s">
         <v>94</v>
       </c>
-      <c r="G24" s="115" t="s">
-        <v>528</v>
-      </c>
-      <c r="H24" s="12"/>
-    </row>
-    <row r="25" spans="1:8" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A25" s="109"/>
-      <c r="B25" s="114" t="s">
+      <c r="G25" s="114" t="s">
+        <v>527</v>
+      </c>
+      <c r="H25" s="12"/>
+    </row>
+    <row r="26" spans="2:8" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="B26" s="113" t="s">
         <v>90</v>
       </c>
-      <c r="C25" s="114" t="s">
+      <c r="C26" s="113" t="s">
         <v>506</v>
       </c>
-      <c r="D25" s="115" t="s">
+      <c r="D26" s="114" t="s">
         <v>511</v>
       </c>
-      <c r="E25" s="115" t="s">
+      <c r="E26" s="114" t="s">
         <v>516</v>
       </c>
-      <c r="F25" s="115" t="s">
+      <c r="F26" s="114" t="s">
         <v>94</v>
       </c>
-      <c r="G25" s="115" t="s">
-        <v>528</v>
-      </c>
-      <c r="H25" s="12"/>
-    </row>
-    <row r="26" spans="1:8" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A26" s="109"/>
-      <c r="B26" s="114" t="s">
+      <c r="G26" s="114" t="s">
+        <v>527</v>
+      </c>
+      <c r="H26" s="12"/>
+    </row>
+    <row r="27" spans="2:8" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="B27" s="113" t="s">
         <v>90</v>
       </c>
-      <c r="C26" s="114" t="s">
+      <c r="C27" s="113" t="s">
         <v>507</v>
       </c>
-      <c r="D26" s="115" t="s">
+      <c r="D27" s="114" t="s">
         <v>512</v>
       </c>
-      <c r="E26" s="115" t="s">
+      <c r="E27" s="114" t="s">
         <v>517</v>
       </c>
-      <c r="F26" s="115" t="s">
+      <c r="F27" s="114" t="s">
         <v>94</v>
       </c>
-      <c r="G26" s="115" t="s">
-        <v>528</v>
-      </c>
-      <c r="H26" s="12"/>
-    </row>
-    <row r="27" spans="1:8" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A27" s="109"/>
-      <c r="B27" s="114" t="s">
-        <v>90</v>
-      </c>
-      <c r="C27" s="114" t="s">
-        <v>508</v>
-      </c>
-      <c r="D27" s="115" t="s">
-        <v>513</v>
-      </c>
-      <c r="E27" s="115" t="s">
-        <v>518</v>
-      </c>
-      <c r="F27" s="115" t="s">
-        <v>94</v>
-      </c>
-      <c r="G27" s="115" t="s">
-        <v>528</v>
+      <c r="G27" s="114" t="s">
+        <v>527</v>
       </c>
       <c r="H27" s="12"/>
     </row>
-    <row r="28" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A28" s="109"/>
-      <c r="B28" s="116" t="s">
+    <row r="28" spans="2:8" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="B28" s="115" t="s">
         <v>107</v>
       </c>
-      <c r="C28" s="116" t="s">
+      <c r="C28" s="115" t="s">
         <v>108</v>
       </c>
       <c r="D28" s="22" t="s">
@@ -3854,15 +3841,15 @@
         <v>111</v>
       </c>
       <c r="G28" s="22" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H28" s="12"/>
     </row>
-    <row r="29" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="B29" s="116" t="s">
+    <row r="29" spans="2:8" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="B29" s="115" t="s">
         <v>107</v>
       </c>
-      <c r="C29" s="116" t="s">
+      <c r="C29" s="115" t="s">
         <v>112</v>
       </c>
       <c r="D29" s="22" t="s">
@@ -3875,15 +3862,15 @@
         <v>115</v>
       </c>
       <c r="G29" s="22" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H29" s="12"/>
     </row>
-    <row r="30" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="B30" s="116" t="s">
+    <row r="30" spans="2:8" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="B30" s="115" t="s">
         <v>107</v>
       </c>
-      <c r="C30" s="116" t="s">
+      <c r="C30" s="115" t="s">
         <v>116</v>
       </c>
       <c r="D30" s="22" t="s">
@@ -3896,15 +3883,15 @@
         <v>119</v>
       </c>
       <c r="G30" s="22" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H30" s="12"/>
     </row>
-    <row r="31" spans="1:8" ht="52.8" x14ac:dyDescent="0.3">
-      <c r="B31" s="117" t="s">
+    <row r="31" spans="2:8" ht="52.8" x14ac:dyDescent="0.3">
+      <c r="B31" s="116" t="s">
         <v>120</v>
       </c>
-      <c r="C31" s="117" t="s">
+      <c r="C31" s="116" t="s">
         <v>121</v>
       </c>
       <c r="D31" s="23" t="s">
@@ -3917,36 +3904,36 @@
         <v>124</v>
       </c>
       <c r="G31" s="23" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H31" s="24"/>
     </row>
-    <row r="32" spans="1:8" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="B32" s="117" t="s">
+    <row r="32" spans="2:8" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="B32" s="116" t="s">
         <v>120</v>
       </c>
-      <c r="C32" s="117" t="s">
+      <c r="C32" s="116" t="s">
         <v>125</v>
       </c>
       <c r="D32" s="23" t="s">
         <v>126</v>
       </c>
       <c r="E32" s="23" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="F32" s="23" t="s">
         <v>127</v>
       </c>
       <c r="G32" s="23" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H32" s="24"/>
     </row>
     <row r="33" spans="1:11" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="B33" s="117" t="s">
+      <c r="B33" s="116" t="s">
         <v>120</v>
       </c>
-      <c r="C33" s="117" t="s">
+      <c r="C33" s="116" t="s">
         <v>128</v>
       </c>
       <c r="D33" s="23" t="s">
@@ -3959,15 +3946,15 @@
         <v>131</v>
       </c>
       <c r="G33" s="23" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H33" s="12"/>
     </row>
     <row r="34" spans="1:11" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="B34" s="117" t="s">
+      <c r="B34" s="116" t="s">
         <v>120</v>
       </c>
-      <c r="C34" s="117" t="s">
+      <c r="C34" s="116" t="s">
         <v>132</v>
       </c>
       <c r="D34" s="23" t="s">
@@ -3980,15 +3967,15 @@
         <v>135</v>
       </c>
       <c r="G34" s="23" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H34" s="10"/>
     </row>
     <row r="35" spans="1:11" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="B35" s="117" t="s">
+      <c r="B35" s="116" t="s">
         <v>120</v>
       </c>
-      <c r="C35" s="117" t="s">
+      <c r="C35" s="116" t="s">
         <v>136</v>
       </c>
       <c r="D35" s="23" t="s">
@@ -4001,15 +3988,15 @@
         <v>139</v>
       </c>
       <c r="G35" s="23" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H35" s="12"/>
     </row>
     <row r="36" spans="1:11" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="B36" s="117" t="s">
+      <c r="B36" s="116" t="s">
         <v>120</v>
       </c>
-      <c r="C36" s="117" t="s">
+      <c r="C36" s="116" t="s">
         <v>140</v>
       </c>
       <c r="D36" s="23" t="s">
@@ -4022,15 +4009,15 @@
         <v>143</v>
       </c>
       <c r="G36" s="23" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H36" s="24"/>
     </row>
     <row r="37" spans="1:11" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="B37" s="117" t="s">
+      <c r="B37" s="116" t="s">
         <v>120</v>
       </c>
-      <c r="C37" s="117" t="s">
+      <c r="C37" s="116" t="s">
         <v>144</v>
       </c>
       <c r="D37" s="23" t="s">
@@ -4043,15 +4030,15 @@
         <v>30</v>
       </c>
       <c r="G37" s="23" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H37" s="12"/>
     </row>
     <row r="38" spans="1:11" ht="52.8" x14ac:dyDescent="0.3">
-      <c r="B38" s="117" t="s">
+      <c r="B38" s="116" t="s">
         <v>120</v>
       </c>
-      <c r="C38" s="117" t="s">
+      <c r="C38" s="116" t="s">
         <v>147</v>
       </c>
       <c r="D38" s="23" t="s">
@@ -4064,88 +4051,88 @@
         <v>150</v>
       </c>
       <c r="G38" s="23" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H38" s="12"/>
     </row>
     <row r="39" spans="1:11" ht="52.8" x14ac:dyDescent="0.3">
       <c r="A39" s="97"/>
-      <c r="B39" s="117" t="s">
+      <c r="B39" s="116" t="s">
         <v>120</v>
       </c>
-      <c r="C39" s="117" t="s">
+      <c r="C39" s="116" t="s">
+        <v>498</v>
+      </c>
+      <c r="D39" s="117" t="s">
         <v>499</v>
       </c>
-      <c r="D39" s="118" t="s">
-        <v>500</v>
-      </c>
-      <c r="E39" s="118" t="s">
-        <v>503</v>
-      </c>
-      <c r="F39" s="118"/>
-      <c r="G39" s="118" t="s">
-        <v>525</v>
+      <c r="E39" s="117" t="s">
+        <v>502</v>
+      </c>
+      <c r="F39" s="117"/>
+      <c r="G39" s="117" t="s">
+        <v>524</v>
       </c>
       <c r="H39" s="12"/>
     </row>
     <row r="40" spans="1:11" ht="52.8" x14ac:dyDescent="0.3">
       <c r="A40" s="97"/>
-      <c r="B40" s="117" t="s">
+      <c r="B40" s="116" t="s">
         <v>120</v>
       </c>
-      <c r="C40" s="119" t="s">
-        <v>501</v>
-      </c>
-      <c r="D40" s="118" t="s">
+      <c r="C40" s="118" t="s">
         <v>500</v>
       </c>
-      <c r="E40" s="118" t="s">
-        <v>503</v>
-      </c>
-      <c r="F40" s="118"/>
-      <c r="G40" s="118" t="s">
-        <v>525</v>
+      <c r="D40" s="117" t="s">
+        <v>499</v>
+      </c>
+      <c r="E40" s="117" t="s">
+        <v>502</v>
+      </c>
+      <c r="F40" s="117"/>
+      <c r="G40" s="117" t="s">
+        <v>524</v>
       </c>
       <c r="H40" s="12"/>
     </row>
     <row r="41" spans="1:11" ht="52.8" x14ac:dyDescent="0.3">
       <c r="A41" s="97"/>
-      <c r="B41" s="117" t="s">
+      <c r="B41" s="116" t="s">
         <v>120</v>
       </c>
-      <c r="C41" s="117" t="s">
+      <c r="C41" s="116" t="s">
+        <v>501</v>
+      </c>
+      <c r="D41" s="117" t="s">
+        <v>499</v>
+      </c>
+      <c r="E41" s="117" t="s">
         <v>502</v>
       </c>
-      <c r="D41" s="118" t="s">
-        <v>500</v>
-      </c>
-      <c r="E41" s="118" t="s">
-        <v>503</v>
-      </c>
-      <c r="F41" s="118"/>
-      <c r="G41" s="118" t="s">
-        <v>525</v>
+      <c r="F41" s="117"/>
+      <c r="G41" s="117" t="s">
+        <v>524</v>
       </c>
       <c r="H41" s="12"/>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="B42" s="26" t="s">
         <v>153</v>
       </c>
       <c r="C42" s="26" t="s">
-        <v>473</v>
-      </c>
-      <c r="D42" s="120" t="s">
+        <v>472</v>
+      </c>
+      <c r="D42" s="119" t="s">
+        <v>475</v>
+      </c>
+      <c r="E42" s="119" t="s">
         <v>476</v>
       </c>
-      <c r="E42" s="120" t="s">
-        <v>477</v>
-      </c>
-      <c r="F42" s="120" t="s">
+      <c r="F42" s="119" t="s">
         <v>50</v>
       </c>
-      <c r="G42" s="120" t="s">
-        <v>525</v>
+      <c r="G42" s="119" t="s">
+        <v>524</v>
       </c>
       <c r="H42" s="24"/>
     </row>
@@ -4154,19 +4141,19 @@
         <v>153</v>
       </c>
       <c r="C43" s="26" t="s">
+        <v>473</v>
+      </c>
+      <c r="D43" s="119" t="s">
         <v>474</v>
       </c>
-      <c r="D43" s="120" t="s">
-        <v>475</v>
-      </c>
-      <c r="E43" s="120" t="s">
-        <v>478</v>
-      </c>
-      <c r="F43" s="120" t="s">
+      <c r="E43" s="119" t="s">
+        <v>477</v>
+      </c>
+      <c r="F43" s="119" t="s">
         <v>152</v>
       </c>
-      <c r="G43" s="120" t="s">
-        <v>525</v>
+      <c r="G43" s="119" t="s">
+        <v>524</v>
       </c>
       <c r="H43" s="24"/>
     </row>
@@ -4175,19 +4162,19 @@
         <v>153</v>
       </c>
       <c r="C44" s="26" t="s">
+        <v>518</v>
+      </c>
+      <c r="D44" s="119" t="s">
         <v>519</v>
       </c>
-      <c r="D44" s="120" t="s">
+      <c r="E44" s="119" t="s">
         <v>520</v>
       </c>
-      <c r="E44" s="120" t="s">
-        <v>521</v>
-      </c>
-      <c r="F44" s="120" t="s">
+      <c r="F44" s="119" t="s">
         <v>152</v>
       </c>
-      <c r="G44" s="120" t="s">
-        <v>526</v>
+      <c r="G44" s="119" t="s">
+        <v>525</v>
       </c>
       <c r="H44" s="24"/>
     </row>
@@ -4196,20 +4183,20 @@
       <c r="B45" s="26" t="s">
         <v>153</v>
       </c>
-      <c r="C45" s="120" t="s">
+      <c r="C45" s="119" t="s">
         <v>154</v>
       </c>
-      <c r="D45" s="120" t="s">
+      <c r="D45" s="119" t="s">
         <v>155</v>
       </c>
-      <c r="E45" s="120" t="s">
+      <c r="E45" s="119" t="s">
         <v>156</v>
       </c>
-      <c r="F45" s="120" t="s">
+      <c r="F45" s="119" t="s">
         <v>157</v>
       </c>
-      <c r="G45" s="120" t="s">
-        <v>525</v>
+      <c r="G45" s="119" t="s">
+        <v>524</v>
       </c>
       <c r="H45" s="30"/>
       <c r="I45" s="28"/>
@@ -4221,20 +4208,20 @@
       <c r="B46" s="26" t="s">
         <v>153</v>
       </c>
-      <c r="C46" s="120" t="s">
+      <c r="C46" s="119" t="s">
         <v>158</v>
       </c>
-      <c r="D46" s="120" t="s">
+      <c r="D46" s="119" t="s">
         <v>159</v>
       </c>
-      <c r="E46" s="120" t="s">
+      <c r="E46" s="119" t="s">
         <v>160</v>
       </c>
       <c r="F46" s="26" t="s">
         <v>152</v>
       </c>
       <c r="G46" s="26" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H46" s="30"/>
       <c r="I46" s="28"/>
@@ -4246,20 +4233,20 @@
       <c r="B47" s="26" t="s">
         <v>153</v>
       </c>
-      <c r="C47" s="120" t="s">
+      <c r="C47" s="119" t="s">
         <v>161</v>
       </c>
-      <c r="D47" s="120" t="s">
+      <c r="D47" s="119" t="s">
         <v>162</v>
       </c>
-      <c r="E47" s="120" t="s">
-        <v>479</v>
-      </c>
-      <c r="F47" s="120" t="s">
+      <c r="E47" s="119" t="s">
+        <v>478</v>
+      </c>
+      <c r="F47" s="119" t="s">
         <v>157</v>
       </c>
-      <c r="G47" s="120" t="s">
-        <v>526</v>
+      <c r="G47" s="119" t="s">
+        <v>525</v>
       </c>
       <c r="H47" s="30"/>
       <c r="I47" s="28"/>
@@ -4271,20 +4258,20 @@
       <c r="B48" s="26" t="s">
         <v>153</v>
       </c>
-      <c r="C48" s="120" t="s">
+      <c r="C48" s="119" t="s">
         <v>163</v>
       </c>
-      <c r="D48" s="120" t="s">
+      <c r="D48" s="119" t="s">
         <v>164</v>
       </c>
-      <c r="E48" s="120" t="s">
-        <v>480</v>
+      <c r="E48" s="119" t="s">
+        <v>479</v>
       </c>
       <c r="F48" s="26" t="s">
         <v>152</v>
       </c>
       <c r="G48" s="26" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H48" s="30"/>
       <c r="I48" s="28"/>
@@ -4296,20 +4283,20 @@
       <c r="B49" s="26" t="s">
         <v>153</v>
       </c>
-      <c r="C49" s="120" t="s">
+      <c r="C49" s="119" t="s">
         <v>165</v>
       </c>
-      <c r="D49" s="120" t="s">
+      <c r="D49" s="119" t="s">
         <v>166</v>
       </c>
-      <c r="E49" s="120" t="s">
-        <v>481</v>
-      </c>
-      <c r="F49" s="120" t="s">
+      <c r="E49" s="119" t="s">
+        <v>480</v>
+      </c>
+      <c r="F49" s="119" t="s">
         <v>157</v>
       </c>
-      <c r="G49" s="120" t="s">
-        <v>526</v>
+      <c r="G49" s="119" t="s">
+        <v>525</v>
       </c>
       <c r="H49" s="30"/>
       <c r="I49" s="28"/>
@@ -4321,20 +4308,20 @@
       <c r="B50" s="26" t="s">
         <v>153</v>
       </c>
-      <c r="C50" s="120" t="s">
+      <c r="C50" s="119" t="s">
         <v>167</v>
       </c>
-      <c r="D50" s="120" t="s">
+      <c r="D50" s="119" t="s">
         <v>168</v>
       </c>
-      <c r="E50" s="120" t="s">
-        <v>482</v>
+      <c r="E50" s="119" t="s">
+        <v>481</v>
       </c>
       <c r="F50" s="26" t="s">
         <v>152</v>
       </c>
       <c r="G50" s="26" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H50" s="30"/>
       <c r="I50" s="28"/>
@@ -4346,20 +4333,20 @@
       <c r="B51" s="26" t="s">
         <v>153</v>
       </c>
-      <c r="C51" s="120" t="s">
+      <c r="C51" s="119" t="s">
         <v>169</v>
       </c>
-      <c r="D51" s="120" t="s">
+      <c r="D51" s="119" t="s">
         <v>170</v>
       </c>
-      <c r="E51" s="120" t="s">
-        <v>483</v>
-      </c>
-      <c r="F51" s="120" t="s">
+      <c r="E51" s="119" t="s">
+        <v>482</v>
+      </c>
+      <c r="F51" s="119" t="s">
         <v>157</v>
       </c>
-      <c r="G51" s="120" t="s">
-        <v>526</v>
+      <c r="G51" s="119" t="s">
+        <v>525</v>
       </c>
       <c r="H51" s="30"/>
       <c r="I51" s="28"/>
@@ -4371,20 +4358,20 @@
       <c r="B52" s="26" t="s">
         <v>153</v>
       </c>
-      <c r="C52" s="120" t="s">
+      <c r="C52" s="119" t="s">
         <v>171</v>
       </c>
-      <c r="D52" s="120" t="s">
+      <c r="D52" s="119" t="s">
         <v>172</v>
       </c>
-      <c r="E52" s="120" t="s">
-        <v>484</v>
+      <c r="E52" s="119" t="s">
+        <v>483</v>
       </c>
       <c r="F52" s="26" t="s">
         <v>152</v>
       </c>
       <c r="G52" s="26" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H52" s="30"/>
       <c r="I52" s="28"/>
@@ -4396,20 +4383,20 @@
       <c r="B53" s="26" t="s">
         <v>153</v>
       </c>
-      <c r="C53" s="120" t="s">
+      <c r="C53" s="119" t="s">
         <v>173</v>
       </c>
-      <c r="D53" s="120" t="s">
+      <c r="D53" s="119" t="s">
         <v>174</v>
       </c>
-      <c r="E53" s="120" t="s">
-        <v>485</v>
-      </c>
-      <c r="F53" s="120" t="s">
+      <c r="E53" s="119" t="s">
+        <v>484</v>
+      </c>
+      <c r="F53" s="119" t="s">
         <v>157</v>
       </c>
-      <c r="G53" s="120" t="s">
-        <v>526</v>
+      <c r="G53" s="119" t="s">
+        <v>525</v>
       </c>
       <c r="H53" s="30"/>
       <c r="I53" s="28"/>
@@ -4421,20 +4408,20 @@
       <c r="B54" s="26" t="s">
         <v>153</v>
       </c>
-      <c r="C54" s="120" t="s">
+      <c r="C54" s="119" t="s">
         <v>175</v>
       </c>
-      <c r="D54" s="120" t="s">
+      <c r="D54" s="119" t="s">
         <v>176</v>
       </c>
-      <c r="E54" s="120" t="s">
-        <v>486</v>
+      <c r="E54" s="119" t="s">
+        <v>485</v>
       </c>
       <c r="F54" s="26" t="s">
         <v>152</v>
       </c>
       <c r="G54" s="26" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H54" s="30"/>
       <c r="I54" s="28"/>
@@ -4446,20 +4433,20 @@
       <c r="B55" s="26" t="s">
         <v>153</v>
       </c>
-      <c r="C55" s="120" t="s">
+      <c r="C55" s="119" t="s">
         <v>177</v>
       </c>
-      <c r="D55" s="120" t="s">
+      <c r="D55" s="119" t="s">
         <v>178</v>
       </c>
-      <c r="E55" s="120" t="s">
-        <v>487</v>
-      </c>
-      <c r="F55" s="120" t="s">
+      <c r="E55" s="119" t="s">
+        <v>486</v>
+      </c>
+      <c r="F55" s="119" t="s">
         <v>157</v>
       </c>
-      <c r="G55" s="120" t="s">
-        <v>526</v>
+      <c r="G55" s="119" t="s">
+        <v>525</v>
       </c>
       <c r="H55" s="30"/>
       <c r="I55" s="28"/>
@@ -4471,20 +4458,20 @@
       <c r="B56" s="26" t="s">
         <v>153</v>
       </c>
-      <c r="C56" s="120" t="s">
+      <c r="C56" s="119" t="s">
         <v>179</v>
       </c>
-      <c r="D56" s="120" t="s">
+      <c r="D56" s="119" t="s">
         <v>180</v>
       </c>
-      <c r="E56" s="120" t="s">
-        <v>488</v>
+      <c r="E56" s="119" t="s">
+        <v>487</v>
       </c>
       <c r="F56" s="26" t="s">
         <v>152</v>
       </c>
       <c r="G56" s="26" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H56" s="30"/>
       <c r="I56" s="28"/>
@@ -4496,20 +4483,20 @@
       <c r="B57" s="26" t="s">
         <v>153</v>
       </c>
-      <c r="C57" s="120" t="s">
+      <c r="C57" s="119" t="s">
         <v>181</v>
       </c>
-      <c r="D57" s="120" t="s">
+      <c r="D57" s="119" t="s">
         <v>182</v>
       </c>
-      <c r="E57" s="120" t="s">
-        <v>489</v>
-      </c>
-      <c r="F57" s="120" t="s">
+      <c r="E57" s="119" t="s">
+        <v>488</v>
+      </c>
+      <c r="F57" s="119" t="s">
         <v>157</v>
       </c>
-      <c r="G57" s="120" t="s">
-        <v>526</v>
+      <c r="G57" s="119" t="s">
+        <v>525</v>
       </c>
       <c r="H57" s="30"/>
       <c r="I57" s="28"/>
@@ -4521,20 +4508,20 @@
       <c r="B58" s="26" t="s">
         <v>153</v>
       </c>
-      <c r="C58" s="120" t="s">
+      <c r="C58" s="119" t="s">
         <v>183</v>
       </c>
-      <c r="D58" s="120" t="s">
+      <c r="D58" s="119" t="s">
         <v>184</v>
       </c>
-      <c r="E58" s="120" t="s">
-        <v>490</v>
+      <c r="E58" s="119" t="s">
+        <v>489</v>
       </c>
       <c r="F58" s="26" t="s">
         <v>152</v>
       </c>
       <c r="G58" s="26" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H58" s="30"/>
       <c r="I58" s="28"/>
@@ -4546,20 +4533,20 @@
       <c r="B59" s="26" t="s">
         <v>153</v>
       </c>
-      <c r="C59" s="120" t="s">
+      <c r="C59" s="119" t="s">
         <v>185</v>
       </c>
-      <c r="D59" s="120" t="s">
+      <c r="D59" s="119" t="s">
         <v>186</v>
       </c>
-      <c r="E59" s="120" t="s">
-        <v>491</v>
-      </c>
-      <c r="F59" s="120" t="s">
+      <c r="E59" s="119" t="s">
+        <v>490</v>
+      </c>
+      <c r="F59" s="119" t="s">
         <v>157</v>
       </c>
-      <c r="G59" s="120" t="s">
-        <v>526</v>
+      <c r="G59" s="119" t="s">
+        <v>525</v>
       </c>
       <c r="H59" s="30"/>
       <c r="I59" s="28"/>
@@ -4571,20 +4558,20 @@
       <c r="B60" s="26" t="s">
         <v>153</v>
       </c>
-      <c r="C60" s="120" t="s">
+      <c r="C60" s="119" t="s">
         <v>187</v>
       </c>
-      <c r="D60" s="120" t="s">
+      <c r="D60" s="119" t="s">
         <v>188</v>
       </c>
-      <c r="E60" s="120" t="s">
-        <v>492</v>
+      <c r="E60" s="119" t="s">
+        <v>491</v>
       </c>
       <c r="F60" s="26" t="s">
         <v>152</v>
       </c>
       <c r="G60" s="26" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H60" s="30"/>
       <c r="I60" s="28"/>
@@ -4596,20 +4583,20 @@
       <c r="B61" s="26" t="s">
         <v>153</v>
       </c>
-      <c r="C61" s="120" t="s">
+      <c r="C61" s="119" t="s">
         <v>189</v>
       </c>
-      <c r="D61" s="120" t="s">
+      <c r="D61" s="119" t="s">
         <v>190</v>
       </c>
-      <c r="E61" s="120" t="s">
-        <v>493</v>
-      </c>
-      <c r="F61" s="120" t="s">
+      <c r="E61" s="119" t="s">
+        <v>492</v>
+      </c>
+      <c r="F61" s="119" t="s">
         <v>157</v>
       </c>
-      <c r="G61" s="120" t="s">
-        <v>526</v>
+      <c r="G61" s="119" t="s">
+        <v>525</v>
       </c>
       <c r="H61" s="30"/>
       <c r="I61" s="28"/>
@@ -4621,20 +4608,20 @@
       <c r="B62" s="26" t="s">
         <v>153</v>
       </c>
-      <c r="C62" s="120" t="s">
+      <c r="C62" s="119" t="s">
         <v>191</v>
       </c>
-      <c r="D62" s="120" t="s">
+      <c r="D62" s="119" t="s">
         <v>192</v>
       </c>
-      <c r="E62" s="120" t="s">
-        <v>494</v>
+      <c r="E62" s="119" t="s">
+        <v>493</v>
       </c>
       <c r="F62" s="26" t="s">
         <v>152</v>
       </c>
       <c r="G62" s="26" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H62" s="30"/>
       <c r="I62" s="28"/>
@@ -4646,20 +4633,20 @@
       <c r="B63" s="26" t="s">
         <v>153</v>
       </c>
-      <c r="C63" s="120" t="s">
+      <c r="C63" s="119" t="s">
         <v>193</v>
       </c>
-      <c r="D63" s="120" t="s">
+      <c r="D63" s="119" t="s">
         <v>194</v>
       </c>
-      <c r="E63" s="120" t="s">
-        <v>495</v>
-      </c>
-      <c r="F63" s="120" t="s">
+      <c r="E63" s="119" t="s">
+        <v>494</v>
+      </c>
+      <c r="F63" s="119" t="s">
         <v>157</v>
       </c>
-      <c r="G63" s="120" t="s">
-        <v>526</v>
+      <c r="G63" s="119" t="s">
+        <v>525</v>
       </c>
       <c r="H63" s="30"/>
       <c r="I63" s="28"/>
@@ -4671,20 +4658,20 @@
       <c r="B64" s="26" t="s">
         <v>153</v>
       </c>
-      <c r="C64" s="120" t="s">
+      <c r="C64" s="119" t="s">
         <v>195</v>
       </c>
-      <c r="D64" s="120" t="s">
+      <c r="D64" s="119" t="s">
         <v>196</v>
       </c>
-      <c r="E64" s="120" t="s">
-        <v>496</v>
+      <c r="E64" s="119" t="s">
+        <v>495</v>
       </c>
       <c r="F64" s="26" t="s">
         <v>152</v>
       </c>
       <c r="G64" s="26" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H64" s="30"/>
       <c r="I64" s="28"/>
@@ -4695,20 +4682,20 @@
       <c r="B65" s="26" t="s">
         <v>153</v>
       </c>
-      <c r="C65" s="120" t="s">
+      <c r="C65" s="119" t="s">
         <v>197</v>
       </c>
-      <c r="D65" s="120" t="s">
+      <c r="D65" s="119" t="s">
         <v>198</v>
       </c>
-      <c r="E65" s="120" t="s">
-        <v>497</v>
-      </c>
-      <c r="F65" s="120" t="s">
+      <c r="E65" s="119" t="s">
+        <v>496</v>
+      </c>
+      <c r="F65" s="119" t="s">
         <v>157</v>
       </c>
-      <c r="G65" s="120" t="s">
-        <v>526</v>
+      <c r="G65" s="119" t="s">
+        <v>525</v>
       </c>
       <c r="H65" s="12"/>
     </row>
@@ -4716,20 +4703,20 @@
       <c r="B66" s="26" t="s">
         <v>153</v>
       </c>
-      <c r="C66" s="120" t="s">
+      <c r="C66" s="119" t="s">
         <v>199</v>
       </c>
-      <c r="D66" s="120" t="s">
+      <c r="D66" s="119" t="s">
         <v>200</v>
       </c>
-      <c r="E66" s="120" t="s">
-        <v>498</v>
+      <c r="E66" s="119" t="s">
+        <v>497</v>
       </c>
       <c r="F66" s="26" t="s">
         <v>152</v>
       </c>
       <c r="G66" s="26" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H66" s="12"/>
     </row>
@@ -4751,7 +4738,7 @@
         <v>151</v>
       </c>
       <c r="G67" s="36" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="H67" s="31"/>
       <c r="I67" s="32"/>
@@ -4776,7 +4763,7 @@
         <v>208</v>
       </c>
       <c r="G68" s="36" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="H68" s="31"/>
       <c r="I68" s="32"/>
@@ -4801,7 +4788,7 @@
         <v>152</v>
       </c>
       <c r="G69" s="36" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="H69" s="31"/>
       <c r="I69" s="32"/>
@@ -4826,7 +4813,7 @@
         <v>215</v>
       </c>
       <c r="G70" s="36" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="H70" s="31"/>
       <c r="I70" s="32"/>
@@ -4845,13 +4832,13 @@
         <v>217</v>
       </c>
       <c r="E71" s="37" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="F71" s="36" t="s">
         <v>218</v>
       </c>
       <c r="G71" s="36" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="H71" s="31"/>
       <c r="I71" s="32"/>
@@ -4876,7 +4863,7 @@
         <v>30</v>
       </c>
       <c r="G72" s="36" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="H72" s="31"/>
       <c r="I72" s="32"/>
@@ -4901,7 +4888,7 @@
         <v>152</v>
       </c>
       <c r="G73" s="36" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="H73" s="31"/>
       <c r="I73" s="32"/>
@@ -4926,7 +4913,7 @@
         <v>228</v>
       </c>
       <c r="G74" s="36" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="H74" s="31"/>
       <c r="I74" s="32"/>
@@ -4945,13 +4932,13 @@
         <v>230</v>
       </c>
       <c r="E75" s="37" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="F75" s="37" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="G75" s="36" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="H75" s="31"/>
       <c r="I75" s="32"/>
@@ -4976,7 +4963,7 @@
         <v>30</v>
       </c>
       <c r="G76" s="36" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="H76" s="31"/>
       <c r="I76" s="32"/>
@@ -5001,7 +4988,7 @@
         <v>152</v>
       </c>
       <c r="G77" s="36" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="H77" s="31"/>
       <c r="I77" s="32"/>
@@ -5026,7 +5013,7 @@
         <v>215</v>
       </c>
       <c r="G78" s="36" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="H78" s="31"/>
       <c r="I78" s="32"/>
@@ -5045,13 +5032,13 @@
         <v>239</v>
       </c>
       <c r="E79" s="37" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="F79" s="36" t="s">
         <v>218</v>
       </c>
       <c r="G79" s="36" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="H79" s="31"/>
       <c r="I79" s="32"/>
@@ -5070,13 +5057,13 @@
         <v>241</v>
       </c>
       <c r="E80" s="37" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="F80" s="37" t="s">
         <v>30</v>
       </c>
       <c r="G80" s="36" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="H80" s="31"/>
       <c r="I80" s="32"/>
@@ -5101,7 +5088,7 @@
         <v>152</v>
       </c>
       <c r="G81" s="36" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="H81" s="31"/>
       <c r="I81" s="32"/>
@@ -5126,7 +5113,7 @@
         <v>228</v>
       </c>
       <c r="G82" s="36" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="H82" s="31"/>
       <c r="I82" s="32"/>
@@ -5144,13 +5131,13 @@
         <v>249</v>
       </c>
       <c r="E83" s="37" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="F83" s="37" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="G83" s="36" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="H83" s="12"/>
     </row>
@@ -5171,7 +5158,7 @@
         <v>30</v>
       </c>
       <c r="G84" s="36" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="H84" s="12"/>
     </row>
@@ -5192,7 +5179,7 @@
         <v>255</v>
       </c>
       <c r="G85" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H85" s="10"/>
     </row>
@@ -5213,7 +5200,7 @@
         <v>152</v>
       </c>
       <c r="G86" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H86" s="12"/>
     </row>
@@ -5235,7 +5222,7 @@
         <v>262</v>
       </c>
       <c r="G87" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H87" s="30"/>
       <c r="I87" s="28"/>
@@ -5260,7 +5247,7 @@
         <v>152</v>
       </c>
       <c r="G88" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H88" s="30"/>
       <c r="I88" s="28"/>
@@ -5285,7 +5272,7 @@
         <v>152</v>
       </c>
       <c r="G89" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H89" s="30"/>
       <c r="I89" s="28"/>
@@ -5310,7 +5297,7 @@
         <v>262</v>
       </c>
       <c r="G90" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H90" s="30"/>
       <c r="I90" s="28"/>
@@ -5335,7 +5322,7 @@
         <v>152</v>
       </c>
       <c r="G91" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H91" s="30"/>
       <c r="I91" s="28"/>
@@ -5360,7 +5347,7 @@
         <v>152</v>
       </c>
       <c r="G92" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H92" s="30"/>
       <c r="I92" s="28"/>
@@ -5372,20 +5359,20 @@
       <c r="B93" s="36" t="s">
         <v>201</v>
       </c>
-      <c r="C93" s="121" t="s">
+      <c r="C93" s="120" t="s">
         <v>278</v>
       </c>
-      <c r="D93" s="121" t="s">
+      <c r="D93" s="120" t="s">
         <v>279</v>
       </c>
-      <c r="E93" s="121" t="s">
+      <c r="E93" s="120" t="s">
         <v>280</v>
       </c>
-      <c r="F93" s="122" t="s">
+      <c r="F93" s="121" t="s">
         <v>152</v>
       </c>
-      <c r="G93" s="122" t="s">
-        <v>526</v>
+      <c r="G93" s="121" t="s">
+        <v>525</v>
       </c>
       <c r="H93" s="30"/>
       <c r="I93" s="28"/>
@@ -5397,20 +5384,20 @@
       <c r="B94" s="36" t="s">
         <v>201</v>
       </c>
-      <c r="C94" s="121" t="s">
+      <c r="C94" s="120" t="s">
         <v>281</v>
       </c>
-      <c r="D94" s="121" t="s">
+      <c r="D94" s="120" t="s">
         <v>282</v>
       </c>
-      <c r="E94" s="121" t="s">
+      <c r="E94" s="120" t="s">
         <v>283</v>
       </c>
-      <c r="F94" s="121" t="s">
+      <c r="F94" s="120" t="s">
         <v>157</v>
       </c>
-      <c r="G94" s="121" t="s">
-        <v>526</v>
+      <c r="G94" s="120" t="s">
+        <v>525</v>
       </c>
       <c r="H94" s="31"/>
       <c r="I94" s="32"/>
@@ -5428,14 +5415,14 @@
       <c r="D95" s="37" t="s">
         <v>285</v>
       </c>
-      <c r="E95" s="121" t="s">
+      <c r="E95" s="120" t="s">
         <v>286</v>
       </c>
       <c r="F95" s="36" t="s">
         <v>152</v>
       </c>
       <c r="G95" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H95" s="31"/>
       <c r="I95" s="32"/>
@@ -5454,13 +5441,13 @@
         <v>288</v>
       </c>
       <c r="E96" s="37" t="s">
+        <v>540</v>
+      </c>
+      <c r="F96" s="36" t="s">
         <v>289</v>
       </c>
-      <c r="F96" s="36" t="s">
-        <v>290</v>
-      </c>
       <c r="G96" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H96" s="31"/>
       <c r="I96" s="32"/>
@@ -5473,19 +5460,19 @@
         <v>201</v>
       </c>
       <c r="C97" s="36" t="s">
+        <v>290</v>
+      </c>
+      <c r="D97" s="37" t="s">
         <v>291</v>
       </c>
-      <c r="D97" s="37" t="s">
+      <c r="E97" s="120" t="s">
         <v>292</v>
-      </c>
-      <c r="E97" s="121" t="s">
-        <v>293</v>
       </c>
       <c r="F97" s="36" t="s">
         <v>152</v>
       </c>
       <c r="G97" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H97" s="31"/>
       <c r="I97" s="32"/>
@@ -5498,19 +5485,19 @@
         <v>201</v>
       </c>
       <c r="C98" s="36" t="s">
+        <v>293</v>
+      </c>
+      <c r="D98" s="37" t="s">
         <v>294</v>
       </c>
-      <c r="D98" s="37" t="s">
+      <c r="E98" s="120" t="s">
         <v>295</v>
       </c>
-      <c r="E98" s="121" t="s">
-        <v>296</v>
-      </c>
       <c r="F98" s="36" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="G98" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H98" s="31"/>
       <c r="I98" s="32"/>
@@ -5523,19 +5510,19 @@
         <v>201</v>
       </c>
       <c r="C99" s="36" t="s">
+        <v>296</v>
+      </c>
+      <c r="D99" s="37" t="s">
         <v>297</v>
       </c>
-      <c r="D99" s="37" t="s">
+      <c r="E99" s="120" t="s">
         <v>298</v>
-      </c>
-      <c r="E99" s="121" t="s">
-        <v>299</v>
       </c>
       <c r="F99" s="36" t="s">
         <v>152</v>
       </c>
       <c r="G99" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H99" s="31"/>
       <c r="I99" s="32"/>
@@ -5548,19 +5535,19 @@
         <v>201</v>
       </c>
       <c r="C100" s="36" t="s">
+        <v>299</v>
+      </c>
+      <c r="D100" s="37" t="s">
         <v>300</v>
       </c>
-      <c r="D100" s="37" t="s">
+      <c r="E100" s="120" t="s">
         <v>301</v>
       </c>
-      <c r="E100" s="121" t="s">
-        <v>302</v>
-      </c>
       <c r="F100" s="36" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="G100" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H100" s="31"/>
       <c r="I100" s="32"/>
@@ -5573,19 +5560,19 @@
         <v>201</v>
       </c>
       <c r="C101" s="36" t="s">
+        <v>302</v>
+      </c>
+      <c r="D101" s="37" t="s">
         <v>303</v>
       </c>
-      <c r="D101" s="37" t="s">
+      <c r="E101" s="120" t="s">
         <v>304</v>
-      </c>
-      <c r="E101" s="121" t="s">
-        <v>305</v>
       </c>
       <c r="F101" s="36" t="s">
         <v>152</v>
       </c>
       <c r="G101" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H101" s="31"/>
       <c r="I101" s="32"/>
@@ -5598,19 +5585,19 @@
         <v>201</v>
       </c>
       <c r="C102" s="36" t="s">
+        <v>305</v>
+      </c>
+      <c r="D102" s="37" t="s">
         <v>306</v>
       </c>
-      <c r="D102" s="37" t="s">
+      <c r="E102" s="120" t="s">
         <v>307</v>
       </c>
-      <c r="E102" s="121" t="s">
-        <v>308</v>
-      </c>
       <c r="F102" s="36" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="G102" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H102" s="31"/>
       <c r="I102" s="32"/>
@@ -5623,19 +5610,19 @@
         <v>201</v>
       </c>
       <c r="C103" s="36" t="s">
+        <v>308</v>
+      </c>
+      <c r="D103" s="37" t="s">
         <v>309</v>
       </c>
-      <c r="D103" s="37" t="s">
+      <c r="E103" s="120" t="s">
         <v>310</v>
-      </c>
-      <c r="E103" s="121" t="s">
-        <v>311</v>
       </c>
       <c r="F103" s="36" t="s">
         <v>152</v>
       </c>
       <c r="G103" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H103" s="31"/>
       <c r="I103" s="32"/>
@@ -5648,19 +5635,19 @@
         <v>201</v>
       </c>
       <c r="C104" s="36" t="s">
+        <v>311</v>
+      </c>
+      <c r="D104" s="37" t="s">
         <v>312</v>
       </c>
-      <c r="D104" s="37" t="s">
+      <c r="E104" s="120" t="s">
         <v>313</v>
       </c>
-      <c r="E104" s="121" t="s">
-        <v>314</v>
-      </c>
       <c r="F104" s="36" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="G104" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H104" s="31"/>
       <c r="I104" s="32"/>
@@ -5673,19 +5660,19 @@
         <v>201</v>
       </c>
       <c r="C105" s="36" t="s">
+        <v>314</v>
+      </c>
+      <c r="D105" s="37" t="s">
         <v>315</v>
       </c>
-      <c r="D105" s="37" t="s">
+      <c r="E105" s="120" t="s">
         <v>316</v>
-      </c>
-      <c r="E105" s="121" t="s">
-        <v>317</v>
       </c>
       <c r="F105" s="36" t="s">
         <v>152</v>
       </c>
       <c r="G105" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H105" s="31"/>
       <c r="I105" s="32"/>
@@ -5698,19 +5685,19 @@
         <v>201</v>
       </c>
       <c r="C106" s="36" t="s">
+        <v>317</v>
+      </c>
+      <c r="D106" s="37" t="s">
         <v>318</v>
       </c>
-      <c r="D106" s="37" t="s">
+      <c r="E106" s="120" t="s">
         <v>319</v>
       </c>
-      <c r="E106" s="121" t="s">
-        <v>320</v>
-      </c>
       <c r="F106" s="36" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="G106" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H106" s="31"/>
       <c r="I106" s="32"/>
@@ -5723,19 +5710,19 @@
         <v>201</v>
       </c>
       <c r="C107" s="36" t="s">
+        <v>320</v>
+      </c>
+      <c r="D107" s="37" t="s">
         <v>321</v>
       </c>
-      <c r="D107" s="37" t="s">
+      <c r="E107" s="120" t="s">
         <v>322</v>
-      </c>
-      <c r="E107" s="121" t="s">
-        <v>323</v>
       </c>
       <c r="F107" s="36" t="s">
         <v>152</v>
       </c>
       <c r="G107" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H107" s="31"/>
       <c r="I107" s="32"/>
@@ -5748,19 +5735,19 @@
         <v>201</v>
       </c>
       <c r="C108" s="36" t="s">
+        <v>323</v>
+      </c>
+      <c r="D108" s="37" t="s">
         <v>324</v>
       </c>
-      <c r="D108" s="37" t="s">
+      <c r="E108" s="120" t="s">
         <v>325</v>
       </c>
-      <c r="E108" s="121" t="s">
-        <v>326</v>
-      </c>
       <c r="F108" s="36" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="G108" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H108" s="31"/>
       <c r="I108" s="32"/>
@@ -5773,19 +5760,19 @@
         <v>201</v>
       </c>
       <c r="C109" s="36" t="s">
+        <v>326</v>
+      </c>
+      <c r="D109" s="37" t="s">
         <v>327</v>
       </c>
-      <c r="D109" s="37" t="s">
+      <c r="E109" s="120" t="s">
         <v>328</v>
-      </c>
-      <c r="E109" s="121" t="s">
-        <v>329</v>
       </c>
       <c r="F109" s="36" t="s">
         <v>152</v>
       </c>
       <c r="G109" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H109" s="31"/>
       <c r="I109" s="32"/>
@@ -5798,19 +5785,19 @@
         <v>201</v>
       </c>
       <c r="C110" s="36" t="s">
+        <v>329</v>
+      </c>
+      <c r="D110" s="37" t="s">
         <v>330</v>
       </c>
-      <c r="D110" s="37" t="s">
+      <c r="E110" s="120" t="s">
         <v>331</v>
       </c>
-      <c r="E110" s="121" t="s">
-        <v>332</v>
-      </c>
       <c r="F110" s="36" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="G110" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H110" s="31"/>
       <c r="I110" s="32"/>
@@ -5823,19 +5810,19 @@
         <v>201</v>
       </c>
       <c r="C111" s="36" t="s">
+        <v>332</v>
+      </c>
+      <c r="D111" s="37" t="s">
         <v>333</v>
       </c>
-      <c r="D111" s="37" t="s">
+      <c r="E111" s="122" t="s">
         <v>334</v>
-      </c>
-      <c r="E111" s="123" t="s">
-        <v>335</v>
       </c>
       <c r="F111" s="36" t="s">
         <v>152</v>
       </c>
       <c r="G111" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H111" s="31"/>
       <c r="I111" s="32"/>
@@ -5848,19 +5835,19 @@
         <v>201</v>
       </c>
       <c r="C112" s="36" t="s">
+        <v>335</v>
+      </c>
+      <c r="D112" s="37" t="s">
         <v>336</v>
       </c>
-      <c r="D112" s="37" t="s">
+      <c r="E112" s="120" t="s">
         <v>337</v>
       </c>
-      <c r="E112" s="121" t="s">
-        <v>338</v>
-      </c>
       <c r="F112" s="36" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="G112" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H112" s="31"/>
       <c r="I112" s="32"/>
@@ -5873,19 +5860,19 @@
         <v>201</v>
       </c>
       <c r="C113" s="36" t="s">
+        <v>338</v>
+      </c>
+      <c r="D113" s="37" t="s">
         <v>339</v>
       </c>
-      <c r="D113" s="37" t="s">
+      <c r="E113" s="122" t="s">
         <v>340</v>
-      </c>
-      <c r="E113" s="123" t="s">
-        <v>341</v>
       </c>
       <c r="F113" s="36" t="s">
         <v>152</v>
       </c>
       <c r="G113" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H113" s="31"/>
       <c r="I113" s="32"/>
@@ -5898,19 +5885,19 @@
         <v>201</v>
       </c>
       <c r="C114" s="36" t="s">
+        <v>341</v>
+      </c>
+      <c r="D114" s="37" t="s">
         <v>342</v>
       </c>
-      <c r="D114" s="37" t="s">
+      <c r="E114" s="120" t="s">
         <v>343</v>
       </c>
-      <c r="E114" s="121" t="s">
-        <v>344</v>
-      </c>
       <c r="F114" s="36" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="G114" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H114" s="31"/>
       <c r="I114" s="32"/>
@@ -5923,19 +5910,19 @@
         <v>201</v>
       </c>
       <c r="C115" s="36" t="s">
+        <v>344</v>
+      </c>
+      <c r="D115" s="37" t="s">
         <v>345</v>
       </c>
-      <c r="D115" s="37" t="s">
+      <c r="E115" s="122" t="s">
         <v>346</v>
-      </c>
-      <c r="E115" s="123" t="s">
-        <v>347</v>
       </c>
       <c r="F115" s="36" t="s">
         <v>152</v>
       </c>
       <c r="G115" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H115" s="31"/>
       <c r="I115" s="32"/>
@@ -5948,19 +5935,19 @@
         <v>201</v>
       </c>
       <c r="C116" s="36" t="s">
+        <v>347</v>
+      </c>
+      <c r="D116" s="37" t="s">
         <v>348</v>
       </c>
-      <c r="D116" s="37" t="s">
+      <c r="E116" s="120" t="s">
         <v>349</v>
       </c>
-      <c r="E116" s="121" t="s">
-        <v>350</v>
-      </c>
       <c r="F116" s="36" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="G116" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H116" s="31"/>
       <c r="I116" s="32"/>
@@ -5973,19 +5960,19 @@
         <v>201</v>
       </c>
       <c r="C117" s="36" t="s">
+        <v>350</v>
+      </c>
+      <c r="D117" s="37" t="s">
         <v>351</v>
       </c>
-      <c r="D117" s="37" t="s">
+      <c r="E117" s="122" t="s">
         <v>352</v>
-      </c>
-      <c r="E117" s="123" t="s">
-        <v>353</v>
       </c>
       <c r="F117" s="36" t="s">
         <v>152</v>
       </c>
       <c r="G117" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H117" s="31"/>
       <c r="I117" s="32"/>
@@ -5998,19 +5985,19 @@
         <v>201</v>
       </c>
       <c r="C118" s="36" t="s">
+        <v>353</v>
+      </c>
+      <c r="D118" s="37" t="s">
         <v>354</v>
       </c>
-      <c r="D118" s="37" t="s">
+      <c r="E118" s="120" t="s">
         <v>355</v>
       </c>
-      <c r="E118" s="121" t="s">
-        <v>356</v>
-      </c>
       <c r="F118" s="36" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="G118" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H118" s="31"/>
       <c r="I118" s="32"/>
@@ -6023,19 +6010,19 @@
         <v>201</v>
       </c>
       <c r="C119" s="36" t="s">
+        <v>356</v>
+      </c>
+      <c r="D119" s="37" t="s">
         <v>357</v>
       </c>
-      <c r="D119" s="37" t="s">
+      <c r="E119" s="122" t="s">
         <v>358</v>
-      </c>
-      <c r="E119" s="123" t="s">
-        <v>359</v>
       </c>
       <c r="F119" s="36" t="s">
         <v>152</v>
       </c>
       <c r="G119" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H119" s="31"/>
       <c r="I119" s="32"/>
@@ -6048,19 +6035,19 @@
         <v>201</v>
       </c>
       <c r="C120" s="36" t="s">
+        <v>359</v>
+      </c>
+      <c r="D120" s="37" t="s">
         <v>360</v>
       </c>
-      <c r="D120" s="37" t="s">
+      <c r="E120" s="120" t="s">
         <v>361</v>
       </c>
-      <c r="E120" s="121" t="s">
-        <v>362</v>
-      </c>
       <c r="F120" s="36" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="G120" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H120" s="31"/>
       <c r="I120" s="32"/>
@@ -6073,19 +6060,19 @@
         <v>201</v>
       </c>
       <c r="C121" s="36" t="s">
+        <v>362</v>
+      </c>
+      <c r="D121" s="37" t="s">
         <v>363</v>
       </c>
-      <c r="D121" s="37" t="s">
+      <c r="E121" s="122" t="s">
         <v>364</v>
-      </c>
-      <c r="E121" s="123" t="s">
-        <v>365</v>
       </c>
       <c r="F121" s="36" t="s">
         <v>152</v>
       </c>
       <c r="G121" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H121" s="31"/>
       <c r="I121" s="32"/>
@@ -6098,19 +6085,19 @@
         <v>201</v>
       </c>
       <c r="C122" s="36" t="s">
+        <v>365</v>
+      </c>
+      <c r="D122" s="37" t="s">
         <v>366</v>
       </c>
-      <c r="D122" s="37" t="s">
+      <c r="E122" s="120" t="s">
         <v>367</v>
       </c>
-      <c r="E122" s="121" t="s">
-        <v>368</v>
-      </c>
       <c r="F122" s="36" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="G122" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H122" s="31"/>
       <c r="I122" s="32"/>
@@ -6123,19 +6110,19 @@
         <v>201</v>
       </c>
       <c r="C123" s="36" t="s">
+        <v>368</v>
+      </c>
+      <c r="D123" s="37" t="s">
         <v>369</v>
       </c>
-      <c r="D123" s="37" t="s">
+      <c r="E123" s="122" t="s">
         <v>370</v>
-      </c>
-      <c r="E123" s="123" t="s">
-        <v>371</v>
       </c>
       <c r="F123" s="36" t="s">
         <v>152</v>
       </c>
       <c r="G123" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H123" s="31"/>
       <c r="I123" s="32"/>
@@ -6148,19 +6135,19 @@
         <v>201</v>
       </c>
       <c r="C124" s="36" t="s">
+        <v>371</v>
+      </c>
+      <c r="D124" s="37" t="s">
         <v>372</v>
       </c>
-      <c r="D124" s="37" t="s">
+      <c r="E124" s="120" t="s">
         <v>373</v>
       </c>
-      <c r="E124" s="121" t="s">
-        <v>374</v>
-      </c>
       <c r="F124" s="36" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="G124" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H124" s="31"/>
       <c r="I124" s="32"/>
@@ -6173,19 +6160,19 @@
         <v>201</v>
       </c>
       <c r="C125" s="36" t="s">
+        <v>374</v>
+      </c>
+      <c r="D125" s="37" t="s">
         <v>375</v>
       </c>
-      <c r="D125" s="37" t="s">
+      <c r="E125" s="122" t="s">
         <v>376</v>
-      </c>
-      <c r="E125" s="123" t="s">
-        <v>377</v>
       </c>
       <c r="F125" s="36" t="s">
         <v>152</v>
       </c>
       <c r="G125" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H125" s="31"/>
       <c r="I125" s="32"/>
@@ -6198,19 +6185,19 @@
         <v>201</v>
       </c>
       <c r="C126" s="36" t="s">
+        <v>377</v>
+      </c>
+      <c r="D126" s="37" t="s">
         <v>378</v>
       </c>
-      <c r="D126" s="37" t="s">
+      <c r="E126" s="120" t="s">
         <v>379</v>
       </c>
-      <c r="E126" s="121" t="s">
-        <v>380</v>
-      </c>
       <c r="F126" s="36" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="G126" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H126" s="31"/>
       <c r="I126" s="32"/>
@@ -6223,19 +6210,19 @@
         <v>201</v>
       </c>
       <c r="C127" s="36" t="s">
+        <v>380</v>
+      </c>
+      <c r="D127" s="37" t="s">
         <v>381</v>
       </c>
-      <c r="D127" s="37" t="s">
+      <c r="E127" s="122" t="s">
         <v>382</v>
-      </c>
-      <c r="E127" s="123" t="s">
-        <v>383</v>
       </c>
       <c r="F127" s="36" t="s">
         <v>152</v>
       </c>
       <c r="G127" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H127" s="31"/>
       <c r="I127" s="32"/>
@@ -6248,19 +6235,19 @@
         <v>201</v>
       </c>
       <c r="C128" s="36" t="s">
+        <v>383</v>
+      </c>
+      <c r="D128" s="37" t="s">
         <v>384</v>
       </c>
-      <c r="D128" s="37" t="s">
+      <c r="E128" s="120" t="s">
         <v>385</v>
       </c>
-      <c r="E128" s="121" t="s">
-        <v>386</v>
-      </c>
       <c r="F128" s="36" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="G128" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H128" s="31"/>
       <c r="I128" s="32"/>
@@ -6273,19 +6260,19 @@
         <v>201</v>
       </c>
       <c r="C129" s="36" t="s">
+        <v>386</v>
+      </c>
+      <c r="D129" s="37" t="s">
         <v>387</v>
       </c>
-      <c r="D129" s="37" t="s">
+      <c r="E129" s="122" t="s">
         <v>388</v>
-      </c>
-      <c r="E129" s="123" t="s">
-        <v>389</v>
       </c>
       <c r="F129" s="36" t="s">
         <v>152</v>
       </c>
       <c r="G129" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H129" s="31"/>
       <c r="I129" s="32"/>
@@ -6298,19 +6285,19 @@
         <v>201</v>
       </c>
       <c r="C130" s="36" t="s">
+        <v>389</v>
+      </c>
+      <c r="D130" s="37" t="s">
         <v>390</v>
       </c>
-      <c r="D130" s="37" t="s">
+      <c r="E130" s="120" t="s">
         <v>391</v>
       </c>
-      <c r="E130" s="121" t="s">
-        <v>392</v>
-      </c>
       <c r="F130" s="36" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="G130" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H130" s="31"/>
       <c r="I130" s="32"/>
@@ -6323,19 +6310,19 @@
         <v>201</v>
       </c>
       <c r="C131" s="36" t="s">
+        <v>392</v>
+      </c>
+      <c r="D131" s="37" t="s">
         <v>393</v>
       </c>
-      <c r="D131" s="37" t="s">
+      <c r="E131" s="122" t="s">
         <v>394</v>
-      </c>
-      <c r="E131" s="123" t="s">
-        <v>395</v>
       </c>
       <c r="F131" s="36" t="s">
         <v>152</v>
       </c>
       <c r="G131" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H131" s="31"/>
       <c r="I131" s="32"/>
@@ -6348,19 +6335,19 @@
         <v>201</v>
       </c>
       <c r="C132" s="36" t="s">
+        <v>395</v>
+      </c>
+      <c r="D132" s="37" t="s">
         <v>396</v>
       </c>
-      <c r="D132" s="37" t="s">
+      <c r="E132" s="120" t="s">
         <v>397</v>
       </c>
-      <c r="E132" s="121" t="s">
-        <v>398</v>
-      </c>
       <c r="F132" s="36" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="G132" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H132" s="31"/>
       <c r="I132" s="32"/>
@@ -6373,19 +6360,19 @@
         <v>201</v>
       </c>
       <c r="C133" s="36" t="s">
+        <v>398</v>
+      </c>
+      <c r="D133" s="37" t="s">
         <v>399</v>
       </c>
-      <c r="D133" s="37" t="s">
+      <c r="E133" s="122" t="s">
         <v>400</v>
-      </c>
-      <c r="E133" s="123" t="s">
-        <v>401</v>
       </c>
       <c r="F133" s="36" t="s">
         <v>152</v>
       </c>
       <c r="G133" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H133" s="31"/>
       <c r="I133" s="38"/>
@@ -6398,19 +6385,19 @@
         <v>201</v>
       </c>
       <c r="C134" s="36" t="s">
+        <v>401</v>
+      </c>
+      <c r="D134" s="37" t="s">
         <v>402</v>
       </c>
-      <c r="D134" s="37" t="s">
+      <c r="E134" s="120" t="s">
         <v>403</v>
       </c>
-      <c r="E134" s="121" t="s">
-        <v>404</v>
-      </c>
       <c r="F134" s="36" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="G134" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H134" s="32"/>
       <c r="I134" s="32"/>
@@ -6423,19 +6410,19 @@
         <v>201</v>
       </c>
       <c r="C135" s="36" t="s">
+        <v>404</v>
+      </c>
+      <c r="D135" s="37" t="s">
         <v>405</v>
       </c>
-      <c r="D135" s="37" t="s">
+      <c r="E135" s="122" t="s">
         <v>406</v>
-      </c>
-      <c r="E135" s="123" t="s">
-        <v>407</v>
       </c>
       <c r="F135" s="36" t="s">
         <v>152</v>
       </c>
       <c r="G135" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H135" s="31"/>
       <c r="I135" s="32"/>
@@ -6448,19 +6435,19 @@
         <v>201</v>
       </c>
       <c r="C136" s="36" t="s">
+        <v>407</v>
+      </c>
+      <c r="D136" s="37" t="s">
         <v>408</v>
       </c>
-      <c r="D136" s="37" t="s">
+      <c r="E136" s="120" t="s">
         <v>409</v>
       </c>
-      <c r="E136" s="121" t="s">
-        <v>410</v>
-      </c>
       <c r="F136" s="36" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="G136" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H136" s="31"/>
       <c r="I136" s="32"/>
@@ -6473,19 +6460,19 @@
         <v>201</v>
       </c>
       <c r="C137" s="36" t="s">
+        <v>410</v>
+      </c>
+      <c r="D137" s="37" t="s">
         <v>411</v>
       </c>
-      <c r="D137" s="37" t="s">
+      <c r="E137" s="122" t="s">
         <v>412</v>
-      </c>
-      <c r="E137" s="123" t="s">
-        <v>413</v>
       </c>
       <c r="F137" s="36" t="s">
         <v>152</v>
       </c>
       <c r="G137" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H137" s="31"/>
       <c r="I137" s="32"/>
@@ -6498,19 +6485,19 @@
         <v>201</v>
       </c>
       <c r="C138" s="36" t="s">
+        <v>413</v>
+      </c>
+      <c r="D138" s="37" t="s">
         <v>414</v>
       </c>
-      <c r="D138" s="37" t="s">
+      <c r="E138" s="120" t="s">
         <v>415</v>
       </c>
-      <c r="E138" s="121" t="s">
-        <v>416</v>
-      </c>
       <c r="F138" s="36" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="G138" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H138" s="31"/>
       <c r="I138" s="32"/>
@@ -6523,19 +6510,19 @@
         <v>201</v>
       </c>
       <c r="C139" s="36" t="s">
+        <v>416</v>
+      </c>
+      <c r="D139" s="37" t="s">
         <v>417</v>
       </c>
-      <c r="D139" s="37" t="s">
+      <c r="E139" s="122" t="s">
         <v>418</v>
-      </c>
-      <c r="E139" s="123" t="s">
-        <v>419</v>
       </c>
       <c r="F139" s="36" t="s">
         <v>152</v>
       </c>
       <c r="G139" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H139" s="31"/>
       <c r="I139" s="32"/>
@@ -6548,19 +6535,19 @@
         <v>201</v>
       </c>
       <c r="C140" s="36" t="s">
+        <v>419</v>
+      </c>
+      <c r="D140" s="37" t="s">
         <v>420</v>
       </c>
-      <c r="D140" s="37" t="s">
+      <c r="E140" s="120" t="s">
         <v>421</v>
       </c>
-      <c r="E140" s="121" t="s">
-        <v>422</v>
-      </c>
       <c r="F140" s="36" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="G140" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H140" s="31"/>
       <c r="I140" s="32"/>
@@ -6573,19 +6560,19 @@
         <v>201</v>
       </c>
       <c r="C141" s="36" t="s">
+        <v>422</v>
+      </c>
+      <c r="D141" s="37" t="s">
         <v>423</v>
       </c>
-      <c r="D141" s="37" t="s">
+      <c r="E141" s="122" t="s">
         <v>424</v>
-      </c>
-      <c r="E141" s="123" t="s">
-        <v>425</v>
       </c>
       <c r="F141" s="36" t="s">
         <v>152</v>
       </c>
       <c r="G141" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H141" s="31"/>
       <c r="I141" s="32"/>
@@ -6598,19 +6585,19 @@
         <v>201</v>
       </c>
       <c r="C142" s="36" t="s">
+        <v>425</v>
+      </c>
+      <c r="D142" s="37" t="s">
         <v>426</v>
       </c>
-      <c r="D142" s="37" t="s">
+      <c r="E142" s="120" t="s">
         <v>427</v>
       </c>
-      <c r="E142" s="121" t="s">
-        <v>428</v>
-      </c>
       <c r="F142" s="36" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="G142" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H142" s="31"/>
       <c r="I142" s="32"/>
@@ -6623,19 +6610,19 @@
         <v>201</v>
       </c>
       <c r="C143" s="36" t="s">
+        <v>428</v>
+      </c>
+      <c r="D143" s="37" t="s">
         <v>429</v>
       </c>
-      <c r="D143" s="37" t="s">
+      <c r="E143" s="122" t="s">
         <v>430</v>
-      </c>
-      <c r="E143" s="123" t="s">
-        <v>431</v>
       </c>
       <c r="F143" s="36" t="s">
         <v>152</v>
       </c>
       <c r="G143" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H143" s="31"/>
       <c r="I143" s="32"/>
@@ -6648,19 +6635,19 @@
         <v>201</v>
       </c>
       <c r="C144" s="36" t="s">
+        <v>431</v>
+      </c>
+      <c r="D144" s="37" t="s">
         <v>432</v>
       </c>
-      <c r="D144" s="37" t="s">
+      <c r="E144" s="120" t="s">
         <v>433</v>
       </c>
-      <c r="E144" s="121" t="s">
-        <v>434</v>
-      </c>
       <c r="F144" s="36" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="G144" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H144" s="31"/>
       <c r="I144" s="32"/>
@@ -6669,23 +6656,23 @@
     </row>
     <row r="145" spans="1:11" s="33" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A145"/>
-      <c r="B145" s="124" t="s">
+      <c r="B145" s="123" t="s">
         <v>201</v>
       </c>
-      <c r="C145" s="125" t="s">
+      <c r="C145" s="124" t="s">
+        <v>434</v>
+      </c>
+      <c r="D145" s="125" t="s">
         <v>435</v>
       </c>
-      <c r="D145" s="126" t="s">
+      <c r="E145" s="126" t="s">
         <v>436</v>
       </c>
-      <c r="E145" s="127" t="s">
-        <v>437</v>
-      </c>
-      <c r="F145" s="125" t="s">
+      <c r="F145" s="124" t="s">
         <v>152</v>
       </c>
       <c r="G145" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H145" s="31"/>
       <c r="I145" s="32"/>
@@ -6694,23 +6681,23 @@
     </row>
     <row r="146" spans="1:11" s="33" customFormat="1" ht="171.6" x14ac:dyDescent="0.3">
       <c r="A146"/>
-      <c r="B146" s="128" t="s">
+      <c r="B146" s="127" t="s">
         <v>201</v>
       </c>
-      <c r="C146" s="129" t="s">
+      <c r="C146" s="128" t="s">
+        <v>437</v>
+      </c>
+      <c r="D146" s="129" t="s">
         <v>438</v>
       </c>
-      <c r="D146" s="130" t="s">
+      <c r="E146" s="130" t="s">
         <v>439</v>
       </c>
-      <c r="E146" s="131" t="s">
-        <v>440</v>
-      </c>
       <c r="F146" s="36" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="G146" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H146" s="31"/>
       <c r="I146" s="32"/>
@@ -6719,23 +6706,23 @@
     </row>
     <row r="147" spans="1:11" s="33" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A147"/>
-      <c r="B147" s="124" t="s">
+      <c r="B147" s="123" t="s">
         <v>201</v>
       </c>
-      <c r="C147" s="125" t="s">
+      <c r="C147" s="124" t="s">
+        <v>440</v>
+      </c>
+      <c r="D147" s="125" t="s">
         <v>441</v>
       </c>
-      <c r="D147" s="126" t="s">
+      <c r="E147" s="126" t="s">
         <v>442</v>
       </c>
-      <c r="E147" s="127" t="s">
-        <v>443</v>
-      </c>
-      <c r="F147" s="125" t="s">
+      <c r="F147" s="124" t="s">
         <v>152</v>
       </c>
       <c r="G147" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H147" s="31"/>
       <c r="I147" s="32"/>
@@ -6744,23 +6731,23 @@
     </row>
     <row r="148" spans="1:11" s="33" customFormat="1" ht="171.6" x14ac:dyDescent="0.3">
       <c r="A148"/>
-      <c r="B148" s="128" t="s">
+      <c r="B148" s="127" t="s">
         <v>201</v>
       </c>
-      <c r="C148" s="129" t="s">
+      <c r="C148" s="128" t="s">
+        <v>443</v>
+      </c>
+      <c r="D148" s="129" t="s">
         <v>444</v>
       </c>
-      <c r="D148" s="130" t="s">
+      <c r="E148" s="130" t="s">
         <v>445</v>
       </c>
-      <c r="E148" s="131" t="s">
-        <v>446</v>
-      </c>
       <c r="F148" s="36" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="G148" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H148" s="31"/>
       <c r="I148" s="32"/>
@@ -6769,23 +6756,23 @@
     </row>
     <row r="149" spans="1:11" s="33" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A149"/>
-      <c r="B149" s="124" t="s">
+      <c r="B149" s="123" t="s">
         <v>201</v>
       </c>
-      <c r="C149" s="125" t="s">
+      <c r="C149" s="124" t="s">
+        <v>446</v>
+      </c>
+      <c r="D149" s="125" t="s">
         <v>447</v>
       </c>
-      <c r="D149" s="126" t="s">
+      <c r="E149" s="126" t="s">
         <v>448</v>
       </c>
-      <c r="E149" s="127" t="s">
-        <v>449</v>
-      </c>
-      <c r="F149" s="125" t="s">
+      <c r="F149" s="124" t="s">
         <v>152</v>
       </c>
       <c r="G149" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H149" s="31"/>
       <c r="I149" s="32"/>
@@ -6794,23 +6781,23 @@
     </row>
     <row r="150" spans="1:11" s="33" customFormat="1" ht="171.6" x14ac:dyDescent="0.3">
       <c r="A150"/>
-      <c r="B150" s="128" t="s">
+      <c r="B150" s="127" t="s">
         <v>201</v>
       </c>
-      <c r="C150" s="129" t="s">
+      <c r="C150" s="128" t="s">
+        <v>449</v>
+      </c>
+      <c r="D150" s="129" t="s">
         <v>450</v>
       </c>
-      <c r="D150" s="130" t="s">
+      <c r="E150" s="130" t="s">
         <v>451</v>
       </c>
-      <c r="E150" s="131" t="s">
-        <v>452</v>
-      </c>
       <c r="F150" s="36" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="G150" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H150" s="31"/>
       <c r="I150" s="32"/>
@@ -6822,19 +6809,19 @@
         <v>201</v>
       </c>
       <c r="C151" s="36" t="s">
+        <v>452</v>
+      </c>
+      <c r="D151" s="37" t="s">
         <v>453</v>
       </c>
-      <c r="D151" s="37" t="s">
+      <c r="E151" s="120" t="s">
+        <v>536</v>
+      </c>
+      <c r="F151" s="36" t="s">
         <v>454</v>
       </c>
-      <c r="E151" s="121" t="s">
-        <v>537</v>
-      </c>
-      <c r="F151" s="36" t="s">
-        <v>455</v>
-      </c>
       <c r="G151" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
     </row>
     <row r="152" spans="1:11" ht="79.2" x14ac:dyDescent="0.3">
@@ -6842,82 +6829,79 @@
         <v>201</v>
       </c>
       <c r="C152" s="36" t="s">
+        <v>455</v>
+      </c>
+      <c r="D152" s="37" t="s">
         <v>456</v>
       </c>
-      <c r="D152" s="37" t="s">
-        <v>457</v>
-      </c>
-      <c r="E152" s="121" t="s">
-        <v>538</v>
+      <c r="E152" s="120" t="s">
+        <v>537</v>
       </c>
       <c r="F152" s="36" t="s">
         <v>152</v>
       </c>
       <c r="G152" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
     </row>
     <row r="153" spans="1:11" ht="105.6" x14ac:dyDescent="0.3">
-      <c r="A153" s="109"/>
       <c r="B153" s="36" t="s">
         <v>201</v>
       </c>
       <c r="C153" s="36" t="s">
+        <v>457</v>
+      </c>
+      <c r="D153" s="37" t="s">
         <v>458</v>
       </c>
-      <c r="D153" s="37" t="s">
+      <c r="E153" s="120" t="s">
+        <v>539</v>
+      </c>
+      <c r="F153" s="36" t="s">
         <v>459</v>
       </c>
-      <c r="E153" s="121" t="s">
-        <v>540</v>
-      </c>
-      <c r="F153" s="36" t="s">
-        <v>460</v>
-      </c>
       <c r="G153" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
     </row>
     <row r="154" spans="1:11" ht="66" x14ac:dyDescent="0.3">
-      <c r="A154" s="109"/>
       <c r="B154" s="36" t="s">
         <v>201</v>
       </c>
       <c r="C154" s="36" t="s">
+        <v>460</v>
+      </c>
+      <c r="D154" s="37" t="s">
         <v>461</v>
       </c>
-      <c r="D154" s="37" t="s">
-        <v>462</v>
-      </c>
-      <c r="E154" s="121" t="s">
-        <v>539</v>
+      <c r="E154" s="120" t="s">
+        <v>538</v>
       </c>
       <c r="F154" s="36" t="s">
         <v>30</v>
       </c>
       <c r="G154" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
     </row>
     <row r="155" spans="1:11" ht="250.8" x14ac:dyDescent="0.3">
-      <c r="A155" s="109"/>
       <c r="B155" s="36" t="s">
         <v>201</v>
       </c>
       <c r="C155" s="36" t="s">
+        <v>462</v>
+      </c>
+      <c r="D155" s="37" t="s">
         <v>463</v>
       </c>
-      <c r="D155" s="37" t="s">
-        <v>464</v>
-      </c>
-      <c r="E155" s="121" t="s">
-        <v>536</v>
+      <c r="E155" s="120" t="s">
+        <v>535</v>
       </c>
       <c r="F155" s="36" t="s">
         <v>30</v>
       </c>
       <c r="G155" s="36" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
     </row>
     <row r="156" spans="1:11" x14ac:dyDescent="0.3">
@@ -7041,19 +7025,19 @@
         <v>104</v>
       </c>
       <c r="V1" s="105" t="s">
+        <v>503</v>
+      </c>
+      <c r="W1" s="105" t="s">
         <v>504</v>
       </c>
-      <c r="W1" s="105" t="s">
+      <c r="X1" s="105" t="s">
         <v>505</v>
       </c>
-      <c r="X1" s="105" t="s">
+      <c r="Y1" s="105" t="s">
         <v>506</v>
       </c>
-      <c r="Y1" s="105" t="s">
+      <c r="Z1" s="105" t="s">
         <v>507</v>
-      </c>
-      <c r="Z1" s="105" t="s">
-        <v>508</v>
       </c>
       <c r="AA1" s="106" t="s">
         <v>108</v>
@@ -7089,22 +7073,22 @@
         <v>147</v>
       </c>
       <c r="AL1" s="106" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="AM1" s="106" t="s">
+        <v>500</v>
+      </c>
+      <c r="AN1" s="106" t="s">
         <v>501</v>
       </c>
-      <c r="AN1" s="106" t="s">
-        <v>502</v>
-      </c>
       <c r="AO1" s="107" t="s">
+        <v>472</v>
+      </c>
+      <c r="AP1" s="107" t="s">
         <v>473</v>
       </c>
-      <c r="AP1" s="107" t="s">
-        <v>474</v>
-      </c>
       <c r="AQ1" s="46" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="AR1" s="46" t="s">
         <v>154</v>
@@ -7194,13 +7178,13 @@
         <v>222</v>
       </c>
       <c r="BU1" s="47" t="s">
+        <v>465</v>
+      </c>
+      <c r="BV1" s="47" t="s">
         <v>466</v>
       </c>
-      <c r="BV1" s="47" t="s">
+      <c r="BW1" s="47" t="s">
         <v>467</v>
-      </c>
-      <c r="BW1" s="47" t="s">
-        <v>468</v>
       </c>
       <c r="BX1" s="47" t="s">
         <v>233</v>
@@ -7218,13 +7202,13 @@
         <v>242</v>
       </c>
       <c r="CC1" s="47" t="s">
+        <v>468</v>
+      </c>
+      <c r="CD1" s="47" t="s">
         <v>469</v>
       </c>
-      <c r="CD1" s="47" t="s">
+      <c r="CE1" s="47" t="s">
         <v>470</v>
-      </c>
-      <c r="CE1" s="47" t="s">
-        <v>471</v>
       </c>
       <c r="CF1" s="47" t="s">
         <v>252</v>
@@ -7263,184 +7247,184 @@
         <v>287</v>
       </c>
       <c r="CR1" s="47" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="CS1" s="47" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="CT1" s="47" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="CU1" s="47" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="CV1" s="47" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="CW1" s="47" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="CX1" s="47" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="CY1" s="47" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="CZ1" s="47" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="DA1" s="47" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="DB1" s="47" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="DC1" s="47" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="DD1" s="47" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="DE1" s="47" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="DF1" s="47" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="DG1" s="47" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="DH1" s="47" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="DI1" s="47" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="DJ1" s="47" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="DK1" s="47" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="DL1" s="47" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="DM1" s="47" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="DN1" s="47" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="DO1" s="47" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="DP1" s="47" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="DQ1" s="47" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="DR1" s="47" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="DS1" s="47" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="DT1" s="47" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="DU1" s="47" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="DV1" s="47" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="DW1" s="47" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="DX1" s="47" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="DY1" s="47" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="DZ1" s="47" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="EA1" s="47" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="EB1" s="47" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="EC1" s="47" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="ED1" s="47" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="EE1" s="47" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="EF1" s="47" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="EG1" s="47" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="EH1" s="47" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="EI1" s="47" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="EJ1" s="47" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="EK1" s="47" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="EL1" s="47" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="EM1" s="47" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="EN1" s="47" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="EO1" s="47" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="EP1" s="47" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="EQ1" s="47" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="ER1" s="47" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="ES1" s="47" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="ET1" s="47" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="EU1" s="47" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="EV1" s="47" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="EW1" s="47" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="EX1" s="107" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="EY1" s="107" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
     </row>
     <row r="2" spans="1:155" x14ac:dyDescent="0.3">
@@ -25555,6 +25539,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="42fbd5e6-b175-407a-a25c-5fc6410bf24f" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="a20b3d4d-24e9-4db7-bf1d-acbd8c10320e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100EE7777BCFCD3E741B5CCCE9A87E98C2C" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="f7fc7590daec4eb8e38e018938a160ca">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="a20b3d4d-24e9-4db7-bf1d-acbd8c10320e" xmlns:ns3="42fbd5e6-b175-407a-a25c-5fc6410bf24f" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="c5ca1b94d4b54616210e83d04e6b3cac" ns2:_="" ns3:_="">
     <xsd:import namespace="a20b3d4d-24e9-4db7-bf1d-acbd8c10320e"/>
@@ -25809,27 +25813,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7E9485EC-5D88-4A1C-961D-0F4FE84359B8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="42fbd5e6-b175-407a-a25c-5fc6410bf24f"/>
+    <ds:schemaRef ds:uri="a20b3d4d-24e9-4db7-bf1d-acbd8c10320e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="42fbd5e6-b175-407a-a25c-5fc6410bf24f" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="a20b3d4d-24e9-4db7-bf1d-acbd8c10320e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{286F673D-E70D-4002-B8F5-CAC95B029A7E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9C9C537E-DFD2-4C38-AC8C-930F122DEFFC}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -25846,23 +25849,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{286F673D-E70D-4002-B8F5-CAC95B029A7E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7E9485EC-5D88-4A1C-961D-0F4FE84359B8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="42fbd5e6-b175-407a-a25c-5fc6410bf24f"/>
-    <ds:schemaRef ds:uri="a20b3d4d-24e9-4db7-bf1d-acbd8c10320e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
fix typo in instructions
</commit_message>
<xml_diff>
--- a/data/ALAI UP Client-level Reporting Tool_short_template_2.26.26.xlsx
+++ b/data/ALAI UP Client-level Reporting Tool_short_template_2.26.26.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kmlab\Desktop\Dashboard\alai_up_local_dashboard\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B43DA1EA-AE37-4646-AE84-1C0CCA526BFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F0C3AAA-1DE0-4CC4-9DFB-FEA32C0E0674}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-9840" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{500E2EE0-B1C5-4ACF-BC67-EDC8BDABD2D7}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{500E2EE0-B1C5-4ACF-BC67-EDC8BDABD2D7}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="3" r:id="rId1"/>
@@ -1682,9 +1682,6 @@
       </rPr>
       <t xml:space="preserve"> Ensure that the site name is consistent for each site.</t>
     </r>
-  </si>
-  <si>
-    <t>The excel sheet provided should be used as a guide for preparing your data. Data can be entered manually, but  extracting data from the eletronic medical record and organizing it into the correct format will be easier and more efficient.</t>
   </si>
   <si>
     <t>Optional or Required?</t>
@@ -1968,6 +1965,9 @@
   <si>
     <t>Dose of client's first iCAB/RPV injection.
 Note: for icab_rpv_shot1_dose, use code 2 for a typical loading dose. The dashboard code assumes that the next dose has an injection interval of 1 month (since it is a loading dose). If the expected interval is not 1 month (e.g. if a patient came from another clinic already on monthly iCAB/RPV, use code 6.</t>
+  </si>
+  <si>
+    <t>The excel sheet provided should be used as a guide for preparing your data. Data can be entered manually, but  extracting data from the electronic medical record and organizing it into the correct format will be easier and more efficient.</t>
   </si>
 </sst>
 </file>
@@ -3122,7 +3122,7 @@
     </row>
     <row r="9" spans="2:2" ht="41.4" x14ac:dyDescent="0.25">
       <c r="B9" s="89" t="s">
-        <v>522</v>
+        <v>540</v>
       </c>
     </row>
     <row r="10" spans="2:2" x14ac:dyDescent="0.25">
@@ -3260,7 +3260,7 @@
         <v>26</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="H1" s="3"/>
       <c r="I1" s="4"/>
@@ -3285,7 +3285,7 @@
         <v>30</v>
       </c>
       <c r="G2" s="110" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="H2" s="7"/>
       <c r="I2" s="8"/>
@@ -3309,7 +3309,7 @@
         <v>30</v>
       </c>
       <c r="G3" s="112" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H3" s="12"/>
       <c r="I3" s="8"/>
@@ -3331,7 +3331,7 @@
         <v>38</v>
       </c>
       <c r="G4" s="16" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="H4" s="12"/>
       <c r="I4" s="8"/>
@@ -3353,7 +3353,7 @@
         <v>42</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H5" s="10"/>
       <c r="I5" s="17"/>
@@ -3375,7 +3375,7 @@
         <v>46</v>
       </c>
       <c r="G6" s="16" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="H6" s="12"/>
     </row>
@@ -3396,7 +3396,7 @@
         <v>50</v>
       </c>
       <c r="G7" s="16" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H7" s="12"/>
     </row>
@@ -3418,7 +3418,7 @@
         <v>54</v>
       </c>
       <c r="G8" s="16" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H8" s="10"/>
       <c r="I8" s="18"/>
@@ -3442,7 +3442,7 @@
         <v>58</v>
       </c>
       <c r="G9" s="16" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H9" s="12"/>
     </row>
@@ -3463,7 +3463,7 @@
         <v>62</v>
       </c>
       <c r="G10" s="16" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H10" s="12"/>
     </row>
@@ -3484,11 +3484,11 @@
         <v>66</v>
       </c>
       <c r="G11" s="16" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H11" s="12"/>
     </row>
-    <row r="12" spans="1:11" ht="39.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="B12" s="15" t="s">
         <v>31</v>
       </c>
@@ -3505,7 +3505,7 @@
         <v>70</v>
       </c>
       <c r="G12" s="16" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H12" s="12"/>
     </row>
@@ -3526,7 +3526,7 @@
         <v>74</v>
       </c>
       <c r="G13" s="16" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H13" s="12"/>
     </row>
@@ -3547,7 +3547,7 @@
         <v>78</v>
       </c>
       <c r="G14" s="16" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H14" s="12"/>
     </row>
@@ -3568,7 +3568,7 @@
         <v>30</v>
       </c>
       <c r="G15" s="16" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H15" s="12"/>
     </row>
@@ -3589,7 +3589,7 @@
         <v>85</v>
       </c>
       <c r="G16" s="16" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="H16" s="20"/>
     </row>
@@ -3610,7 +3610,7 @@
         <v>89</v>
       </c>
       <c r="G17" s="16" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H17" s="12"/>
     </row>
@@ -3631,7 +3631,7 @@
         <v>94</v>
       </c>
       <c r="G18" s="114" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="H18" s="12"/>
     </row>
@@ -3652,7 +3652,7 @@
         <v>94</v>
       </c>
       <c r="G19" s="114" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="H19" s="12"/>
     </row>
@@ -3673,7 +3673,7 @@
         <v>94</v>
       </c>
       <c r="G20" s="114" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="H20" s="12"/>
     </row>
@@ -3694,7 +3694,7 @@
         <v>94</v>
       </c>
       <c r="G21" s="114" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="H21" s="12"/>
     </row>
@@ -3715,7 +3715,7 @@
         <v>94</v>
       </c>
       <c r="G22" s="114" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="H22" s="12"/>
     </row>
@@ -3736,7 +3736,7 @@
         <v>94</v>
       </c>
       <c r="G23" s="114" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="H23" s="12"/>
     </row>
@@ -3757,7 +3757,7 @@
         <v>94</v>
       </c>
       <c r="G24" s="114" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="H24" s="12"/>
     </row>
@@ -3778,7 +3778,7 @@
         <v>94</v>
       </c>
       <c r="G25" s="114" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="H25" s="12"/>
     </row>
@@ -3799,7 +3799,7 @@
         <v>94</v>
       </c>
       <c r="G26" s="114" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="H26" s="12"/>
     </row>
@@ -3820,7 +3820,7 @@
         <v>94</v>
       </c>
       <c r="G27" s="114" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="H27" s="12"/>
     </row>
@@ -3841,7 +3841,7 @@
         <v>111</v>
       </c>
       <c r="G28" s="22" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="H28" s="12"/>
     </row>
@@ -3862,7 +3862,7 @@
         <v>115</v>
       </c>
       <c r="G29" s="22" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="H29" s="12"/>
     </row>
@@ -3883,7 +3883,7 @@
         <v>119</v>
       </c>
       <c r="G30" s="22" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="H30" s="12"/>
     </row>
@@ -3904,7 +3904,7 @@
         <v>124</v>
       </c>
       <c r="G31" s="23" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H31" s="24"/>
     </row>
@@ -3919,13 +3919,13 @@
         <v>126</v>
       </c>
       <c r="E32" s="23" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="F32" s="23" t="s">
         <v>127</v>
       </c>
       <c r="G32" s="23" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="H32" s="24"/>
     </row>
@@ -3946,7 +3946,7 @@
         <v>131</v>
       </c>
       <c r="G33" s="23" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="H33" s="12"/>
     </row>
@@ -3967,7 +3967,7 @@
         <v>135</v>
       </c>
       <c r="G34" s="23" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="H34" s="10"/>
     </row>
@@ -3988,7 +3988,7 @@
         <v>139</v>
       </c>
       <c r="G35" s="23" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="H35" s="12"/>
     </row>
@@ -4009,7 +4009,7 @@
         <v>143</v>
       </c>
       <c r="G36" s="23" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="H36" s="24"/>
     </row>
@@ -4030,7 +4030,7 @@
         <v>30</v>
       </c>
       <c r="G37" s="23" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="H37" s="12"/>
     </row>
@@ -4051,7 +4051,7 @@
         <v>150</v>
       </c>
       <c r="G38" s="23" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="H38" s="12"/>
     </row>
@@ -4071,7 +4071,7 @@
       </c>
       <c r="F39" s="117"/>
       <c r="G39" s="117" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="H39" s="12"/>
     </row>
@@ -4091,7 +4091,7 @@
       </c>
       <c r="F40" s="117"/>
       <c r="G40" s="117" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="H40" s="12"/>
     </row>
@@ -4111,11 +4111,11 @@
       </c>
       <c r="F41" s="117"/>
       <c r="G41" s="117" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="H41" s="12"/>
     </row>
-    <row r="42" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B42" s="26" t="s">
         <v>153</v>
       </c>
@@ -4132,7 +4132,7 @@
         <v>50</v>
       </c>
       <c r="G42" s="119" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="H42" s="24"/>
     </row>
@@ -4153,7 +4153,7 @@
         <v>152</v>
       </c>
       <c r="G43" s="119" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="H43" s="24"/>
     </row>
@@ -4174,7 +4174,7 @@
         <v>152</v>
       </c>
       <c r="G44" s="119" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H44" s="24"/>
     </row>
@@ -4196,7 +4196,7 @@
         <v>157</v>
       </c>
       <c r="G45" s="119" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="H45" s="30"/>
       <c r="I45" s="28"/>
@@ -4221,7 +4221,7 @@
         <v>152</v>
       </c>
       <c r="G46" s="26" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="H46" s="30"/>
       <c r="I46" s="28"/>
@@ -4246,7 +4246,7 @@
         <v>157</v>
       </c>
       <c r="G47" s="119" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H47" s="30"/>
       <c r="I47" s="28"/>
@@ -4271,7 +4271,7 @@
         <v>152</v>
       </c>
       <c r="G48" s="26" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H48" s="30"/>
       <c r="I48" s="28"/>
@@ -4296,7 +4296,7 @@
         <v>157</v>
       </c>
       <c r="G49" s="119" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H49" s="30"/>
       <c r="I49" s="28"/>
@@ -4321,7 +4321,7 @@
         <v>152</v>
       </c>
       <c r="G50" s="26" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H50" s="30"/>
       <c r="I50" s="28"/>
@@ -4346,7 +4346,7 @@
         <v>157</v>
       </c>
       <c r="G51" s="119" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H51" s="30"/>
       <c r="I51" s="28"/>
@@ -4371,7 +4371,7 @@
         <v>152</v>
       </c>
       <c r="G52" s="26" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H52" s="30"/>
       <c r="I52" s="28"/>
@@ -4396,7 +4396,7 @@
         <v>157</v>
       </c>
       <c r="G53" s="119" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H53" s="30"/>
       <c r="I53" s="28"/>
@@ -4421,7 +4421,7 @@
         <v>152</v>
       </c>
       <c r="G54" s="26" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H54" s="30"/>
       <c r="I54" s="28"/>
@@ -4446,7 +4446,7 @@
         <v>157</v>
       </c>
       <c r="G55" s="119" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H55" s="30"/>
       <c r="I55" s="28"/>
@@ -4471,7 +4471,7 @@
         <v>152</v>
       </c>
       <c r="G56" s="26" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H56" s="30"/>
       <c r="I56" s="28"/>
@@ -4496,7 +4496,7 @@
         <v>157</v>
       </c>
       <c r="G57" s="119" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H57" s="30"/>
       <c r="I57" s="28"/>
@@ -4521,7 +4521,7 @@
         <v>152</v>
       </c>
       <c r="G58" s="26" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H58" s="30"/>
       <c r="I58" s="28"/>
@@ -4546,7 +4546,7 @@
         <v>157</v>
       </c>
       <c r="G59" s="119" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H59" s="30"/>
       <c r="I59" s="28"/>
@@ -4571,7 +4571,7 @@
         <v>152</v>
       </c>
       <c r="G60" s="26" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H60" s="30"/>
       <c r="I60" s="28"/>
@@ -4596,7 +4596,7 @@
         <v>157</v>
       </c>
       <c r="G61" s="119" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H61" s="30"/>
       <c r="I61" s="28"/>
@@ -4621,7 +4621,7 @@
         <v>152</v>
       </c>
       <c r="G62" s="26" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H62" s="30"/>
       <c r="I62" s="28"/>
@@ -4646,7 +4646,7 @@
         <v>157</v>
       </c>
       <c r="G63" s="119" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H63" s="30"/>
       <c r="I63" s="28"/>
@@ -4671,7 +4671,7 @@
         <v>152</v>
       </c>
       <c r="G64" s="26" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H64" s="30"/>
       <c r="I64" s="28"/>
@@ -4695,7 +4695,7 @@
         <v>157</v>
       </c>
       <c r="G65" s="119" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H65" s="12"/>
     </row>
@@ -4716,7 +4716,7 @@
         <v>152</v>
       </c>
       <c r="G66" s="26" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H66" s="12"/>
     </row>
@@ -4738,7 +4738,7 @@
         <v>151</v>
       </c>
       <c r="G67" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H67" s="31"/>
       <c r="I67" s="32"/>
@@ -4763,7 +4763,7 @@
         <v>208</v>
       </c>
       <c r="G68" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H68" s="31"/>
       <c r="I68" s="32"/>
@@ -4788,7 +4788,7 @@
         <v>152</v>
       </c>
       <c r="G69" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H69" s="31"/>
       <c r="I69" s="32"/>
@@ -4813,7 +4813,7 @@
         <v>215</v>
       </c>
       <c r="G70" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H70" s="31"/>
       <c r="I70" s="32"/>
@@ -4832,13 +4832,13 @@
         <v>217</v>
       </c>
       <c r="E71" s="37" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="F71" s="36" t="s">
         <v>218</v>
       </c>
       <c r="G71" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H71" s="31"/>
       <c r="I71" s="32"/>
@@ -4863,7 +4863,7 @@
         <v>30</v>
       </c>
       <c r="G72" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H72" s="31"/>
       <c r="I72" s="32"/>
@@ -4888,7 +4888,7 @@
         <v>152</v>
       </c>
       <c r="G73" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H73" s="31"/>
       <c r="I73" s="32"/>
@@ -4913,7 +4913,7 @@
         <v>228</v>
       </c>
       <c r="G74" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H74" s="31"/>
       <c r="I74" s="32"/>
@@ -4932,13 +4932,13 @@
         <v>230</v>
       </c>
       <c r="E75" s="37" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="F75" s="37" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="G75" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H75" s="31"/>
       <c r="I75" s="32"/>
@@ -4963,7 +4963,7 @@
         <v>30</v>
       </c>
       <c r="G76" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H76" s="31"/>
       <c r="I76" s="32"/>
@@ -4988,7 +4988,7 @@
         <v>152</v>
       </c>
       <c r="G77" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H77" s="31"/>
       <c r="I77" s="32"/>
@@ -5013,7 +5013,7 @@
         <v>215</v>
       </c>
       <c r="G78" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H78" s="31"/>
       <c r="I78" s="32"/>
@@ -5032,13 +5032,13 @@
         <v>239</v>
       </c>
       <c r="E79" s="37" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="F79" s="36" t="s">
         <v>218</v>
       </c>
       <c r="G79" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H79" s="31"/>
       <c r="I79" s="32"/>
@@ -5057,13 +5057,13 @@
         <v>241</v>
       </c>
       <c r="E80" s="37" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="F80" s="37" t="s">
         <v>30</v>
       </c>
       <c r="G80" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H80" s="31"/>
       <c r="I80" s="32"/>
@@ -5088,7 +5088,7 @@
         <v>152</v>
       </c>
       <c r="G81" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H81" s="31"/>
       <c r="I81" s="32"/>
@@ -5113,7 +5113,7 @@
         <v>228</v>
       </c>
       <c r="G82" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H82" s="31"/>
       <c r="I82" s="32"/>
@@ -5131,13 +5131,13 @@
         <v>249</v>
       </c>
       <c r="E83" s="37" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="F83" s="37" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="G83" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H83" s="12"/>
     </row>
@@ -5158,7 +5158,7 @@
         <v>30</v>
       </c>
       <c r="G84" s="36" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H84" s="12"/>
     </row>
@@ -5179,7 +5179,7 @@
         <v>255</v>
       </c>
       <c r="G85" s="36" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H85" s="10"/>
     </row>
@@ -5200,7 +5200,7 @@
         <v>152</v>
       </c>
       <c r="G86" s="36" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H86" s="12"/>
     </row>
@@ -5222,7 +5222,7 @@
         <v>262</v>
       </c>
       <c r="G87" s="36" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H87" s="30"/>
       <c r="I87" s="28"/>
@@ -5247,7 +5247,7 @@
         <v>152</v>
       </c>
       <c r="G88" s="36" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H88" s="30"/>
       <c r="I88" s="28"/>
@@ -5272,7 +5272,7 @@
         <v>152</v>
       </c>
       <c r="G89" s="36" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H89" s="30"/>
       <c r="I89" s="28"/>
@@ -5297,7 +5297,7 @@
         <v>262</v>
       </c>
       <c r="G90" s="36" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H90" s="30"/>
       <c r="I90" s="28"/>
@@ -5322,7 +5322,7 @@
         <v>152</v>
       </c>
       <c r="G91" s="36" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H91" s="30"/>
       <c r="I91" s="28"/>
@@ -5347,7 +5347,7 @@
         <v>152</v>
       </c>
       <c r="G92" s="36" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H92" s="30"/>
       <c r="I92" s="28"/>
@@ -5372,7 +5372,7 @@
         <v>152</v>
       </c>
       <c r="G93" s="121" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H93" s="30"/>
       <c r="I93" s="28"/>
@@ -5397,7 +5397,7 @@
         <v>157</v>
       </c>
       <c r="G94" s="120" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H94" s="31"/>
       <c r="I94" s="32"/>
@@ -5422,7 +5422,7 @@
         <v>152</v>
       </c>
       <c r="G95" s="36" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H95" s="31"/>
       <c r="I95" s="32"/>
@@ -5441,13 +5441,13 @@
         <v>288</v>
       </c>
       <c r="E96" s="37" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="F96" s="36" t="s">
         <v>289</v>
       </c>
       <c r="G96" s="36" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H96" s="31"/>
       <c r="I96" s="32"/>
@@ -5472,7 +5472,7 @@
         <v>152</v>
       </c>
       <c r="G97" s="36" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H97" s="31"/>
       <c r="I97" s="32"/>
@@ -5497,7 +5497,7 @@
         <v>289</v>
       </c>
       <c r="G98" s="36" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H98" s="31"/>
       <c r="I98" s="32"/>
@@ -5522,7 +5522,7 @@
         <v>152</v>
       </c>
       <c r="G99" s="36" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H99" s="31"/>
       <c r="I99" s="32"/>
@@ -5547,7 +5547,7 @@
         <v>289</v>
       </c>
       <c r="G100" s="36" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H100" s="31"/>
       <c r="I100" s="32"/>
@@ -5572,7 +5572,7 @@
         <v>152</v>
       </c>
       <c r="G101" s="36" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H101" s="31"/>
       <c r="I101" s="32"/>
@@ -5597,7 +5597,7 @@
         <v>289</v>
       </c>
       <c r="G102" s="36" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H102" s="31"/>
       <c r="I102" s="32"/>
@@ -5622,7 +5622,7 @@
         <v>152</v>
       </c>
       <c r="G103" s="36" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H103" s="31"/>
       <c r="I103" s="32"/>
@@ -5647,7 +5647,7 @@
         <v>289</v>
       </c>
       <c r="G104" s="36" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H104" s="31"/>
       <c r="I104" s="32"/>
@@ -5672,7 +5672,7 @@
         <v>152</v>
       </c>
       <c r="G105" s="36" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H105" s="31"/>
       <c r="I105" s="32"/>
@@ -5697,7 +5697,7 @@
         <v>289</v>
       </c>
       <c r="G106" s="36" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H106" s="31"/>
       <c r="I106" s="32"/>
@@ -5722,7 +5722,7 @@
         <v>152</v>
       </c>
       <c r="G107" s="36" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H107" s="31"/>
       <c r="I107" s="32"/>
@@ -5747,7 +5747,7 @@
         <v>289</v>
       </c>
       <c r="G108" s="36" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H108" s="31"/>
       <c r="I108" s="32"/>
@@ -5772,7 +5772,7 @@
         <v>152</v>
       </c>
       <c r="G109" s="36" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H109" s="31"/>
       <c r="I109" s="32"/>
@@ -5797,7 +5797,7 @@
         <v>289</v>
       </c>
       <c r="G110" s="36" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H110" s="31"/>
       <c r="I110" s="32"/>
@@ -5822,7 +5822,7 @@
         <v>152</v>
       </c>
       <c r="G111" s="36" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H111" s="31"/>
       <c r="I111" s="32"/>
@@ -5847,7 +5847,7 @@
         <v>289</v>
       </c>
       <c r="G112" s="36" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H112" s="31"/>
       <c r="I112" s="32"/>
@@ -5872,7 +5872,7 @@
         <v>152</v>
       </c>
       <c r="G113" s="36" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H113" s="31"/>
       <c r="I113" s="32"/>
@@ -5897,7 +5897,7 @@
         <v>289</v>
       </c>
       <c r="G114" s="36" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H114" s="31"/>
       <c r="I114" s="32"/>
@@ -5922,7 +5922,7 @@
         <v>152</v>
       </c>
       <c r="G115" s="36" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H115" s="31"/>
       <c r="I115" s="32"/>
@@ -5947,7 +5947,7 @@
         <v>289</v>
       </c>
       <c r="G116" s="36" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H116" s="31"/>
       <c r="I116" s="32"/>
@@ -5972,7 +5972,7 @@
         <v>152</v>
       </c>
       <c r="G117" s="36" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H117" s="31"/>
       <c r="I117" s="32"/>
@@ -5997,7 +5997,7 @@
         <v>289</v>
       </c>
       <c r="G118" s="36" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H118" s="31"/>
       <c r="I118" s="32"/>
@@ -6022,7 +6022,7 @@
         <v>152</v>
       </c>
       <c r="G119" s="36" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H119" s="31"/>
       <c r="I119" s="32"/>
@@ -6047,7 +6047,7 @@
         <v>289</v>
       </c>
       <c r="G120" s="36" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H120" s="31"/>
       <c r="I120" s="32"/>
@@ -6072,7 +6072,7 @@
         <v>152</v>
       </c>
       <c r="G121" s="36" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H121" s="31"/>
       <c r="I121" s="32"/>
@@ -6097,7 +6097,7 @@
         <v>289</v>
       </c>
       <c r="G122" s="36" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H122" s="31"/>
       <c r="I122" s="32"/>
@@ -6122,7 +6122,7 @@
         <v>152</v>
       </c>
       <c r="G123" s="36" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H123" s="31"/>
       <c r="I123" s="32"/>
@@ -6147,7 +6147,7 @@
         <v>289</v>
       </c>
       <c r="G124" s="36" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H124" s="31"/>
       <c r="I124" s="32"/>
@@ -6172,7 +6172,7 @@
         <v>152</v>
       </c>
       <c r="G125" s="36" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H125" s="31"/>
       <c r="I125" s="32"/>
@@ -6197,7 +6197,7 @@
         <v>289</v>
       </c>
       <c r="G126" s="36" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H126" s="31"/>
       <c r="I126" s="32"/>
@@ -6222,7 +6222,7 @@
         <v>152</v>
       </c>
       <c r="G127" s="36" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H127" s="31"/>
       <c r="I127" s="32"/>
@@ -6247,7 +6247,7 @@
         <v>289</v>
       </c>
       <c r="G128" s="36" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H128" s="31"/>
       <c r="I128" s="32"/>
@@ -6272,7 +6272,7 @@
         <v>152</v>
       </c>
       <c r="G129" s="36" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H129" s="31"/>
       <c r="I129" s="32"/>
@@ -6297,7 +6297,7 @@
         <v>289</v>
       </c>
       <c r="G130" s="36" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H130" s="31"/>
       <c r="I130" s="32"/>
@@ -6322,7 +6322,7 @@
         <v>152</v>
       </c>
       <c r="G131" s="36" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H131" s="31"/>
       <c r="I131" s="32"/>
@@ -6347,7 +6347,7 @@
         <v>289</v>
       </c>
       <c r="G132" s="36" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H132" s="31"/>
       <c r="I132" s="32"/>
@@ -6372,7 +6372,7 @@
         <v>152</v>
       </c>
       <c r="G133" s="36" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H133" s="31"/>
       <c r="I133" s="38"/>
@@ -6397,7 +6397,7 @@
         <v>289</v>
       </c>
       <c r="G134" s="36" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H134" s="32"/>
       <c r="I134" s="32"/>
@@ -6422,7 +6422,7 @@
         <v>152</v>
       </c>
       <c r="G135" s="36" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H135" s="31"/>
       <c r="I135" s="32"/>
@@ -6447,7 +6447,7 @@
         <v>289</v>
       </c>
       <c r="G136" s="36" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H136" s="31"/>
       <c r="I136" s="32"/>
@@ -6472,7 +6472,7 @@
         <v>152</v>
       </c>
       <c r="G137" s="36" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H137" s="31"/>
       <c r="I137" s="32"/>
@@ -6497,7 +6497,7 @@
         <v>289</v>
       </c>
       <c r="G138" s="36" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H138" s="31"/>
       <c r="I138" s="32"/>
@@ -6522,7 +6522,7 @@
         <v>152</v>
       </c>
       <c r="G139" s="36" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H139" s="31"/>
       <c r="I139" s="32"/>
@@ -6547,7 +6547,7 @@
         <v>289</v>
       </c>
       <c r="G140" s="36" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H140" s="31"/>
       <c r="I140" s="32"/>
@@ -6572,7 +6572,7 @@
         <v>152</v>
       </c>
       <c r="G141" s="36" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H141" s="31"/>
       <c r="I141" s="32"/>
@@ -6597,7 +6597,7 @@
         <v>289</v>
       </c>
       <c r="G142" s="36" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H142" s="31"/>
       <c r="I142" s="32"/>
@@ -6622,7 +6622,7 @@
         <v>152</v>
       </c>
       <c r="G143" s="36" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H143" s="31"/>
       <c r="I143" s="32"/>
@@ -6647,7 +6647,7 @@
         <v>289</v>
       </c>
       <c r="G144" s="36" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H144" s="31"/>
       <c r="I144" s="32"/>
@@ -6672,7 +6672,7 @@
         <v>152</v>
       </c>
       <c r="G145" s="36" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H145" s="31"/>
       <c r="I145" s="32"/>
@@ -6697,7 +6697,7 @@
         <v>289</v>
       </c>
       <c r="G146" s="36" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H146" s="31"/>
       <c r="I146" s="32"/>
@@ -6722,7 +6722,7 @@
         <v>152</v>
       </c>
       <c r="G147" s="36" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H147" s="31"/>
       <c r="I147" s="32"/>
@@ -6747,7 +6747,7 @@
         <v>289</v>
       </c>
       <c r="G148" s="36" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H148" s="31"/>
       <c r="I148" s="32"/>
@@ -6772,7 +6772,7 @@
         <v>152</v>
       </c>
       <c r="G149" s="36" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H149" s="31"/>
       <c r="I149" s="32"/>
@@ -6797,7 +6797,7 @@
         <v>289</v>
       </c>
       <c r="G150" s="36" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H150" s="31"/>
       <c r="I150" s="32"/>
@@ -6815,13 +6815,13 @@
         <v>453</v>
       </c>
       <c r="E151" s="120" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="F151" s="36" t="s">
         <v>454</v>
       </c>
       <c r="G151" s="36" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
     </row>
     <row r="152" spans="1:11" ht="79.2" x14ac:dyDescent="0.3">
@@ -6835,13 +6835,13 @@
         <v>456</v>
       </c>
       <c r="E152" s="120" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="F152" s="36" t="s">
         <v>152</v>
       </c>
       <c r="G152" s="36" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
     </row>
     <row r="153" spans="1:11" ht="105.6" x14ac:dyDescent="0.3">
@@ -6855,13 +6855,13 @@
         <v>458</v>
       </c>
       <c r="E153" s="120" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="F153" s="36" t="s">
         <v>459</v>
       </c>
       <c r="G153" s="36" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
     </row>
     <row r="154" spans="1:11" ht="66" x14ac:dyDescent="0.3">
@@ -6875,13 +6875,13 @@
         <v>461</v>
       </c>
       <c r="E154" s="120" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="F154" s="36" t="s">
         <v>30</v>
       </c>
       <c r="G154" s="36" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
     </row>
     <row r="155" spans="1:11" ht="250.8" x14ac:dyDescent="0.3">
@@ -6895,13 +6895,13 @@
         <v>463</v>
       </c>
       <c r="E155" s="120" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="F155" s="36" t="s">
         <v>30</v>
       </c>
       <c r="G155" s="36" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
     </row>
     <row r="156" spans="1:11" x14ac:dyDescent="0.3">
@@ -25539,6 +25539,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="42fbd5e6-b175-407a-a25c-5fc6410bf24f" xsi:nil="true"/>
@@ -25547,15 +25556,6 @@
     </lcf76f155ced4ddcb4097134ff3c332f>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -25814,20 +25814,20 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{286F673D-E70D-4002-B8F5-CAC95B029A7E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7E9485EC-5D88-4A1C-961D-0F4FE84359B8}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="42fbd5e6-b175-407a-a25c-5fc6410bf24f"/>
     <ds:schemaRef ds:uri="a20b3d4d-24e9-4db7-bf1d-acbd8c10320e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{286F673D-E70D-4002-B8F5-CAC95B029A7E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>